<commit_message>
Paso 6: fix parser K91PASEO→K91 y CN37→BS37, regenerar reporte cotizaciones
- canonical_code: strip trailing non-numeric suffix (K91PASEO → K91)
- canonical_code: CN → BS (Cinnabon = Baskin, misma ubicación)
- Resultado final: 153 archivos, 76 OK, 48 inconsistencias, 29 sin match DB

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/REVISION_COTIZACIONES_2026.xlsx
+++ b/REVISION_COTIZACIONES_2026.xlsx
@@ -2095,38 +2095,46 @@
       <c r="J39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>COTIZACION1294 KFCK91PASEO SHOPP MACHALA.xlsx</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>K91PASEO</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="4" t="n">
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>K91</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>K091 - MACHALA RIO CENTRO</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
         <v>87.5</v>
       </c>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="inlineStr"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>SIN_MATCH_DB</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>Codigo 'K91PASEO' no encontrado en DB.</t>
-        </is>
-      </c>
+      <c r="F40" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>173.44</v>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>INCONSISTENCIA</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2525,38 +2533,46 @@
       <c r="J50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1359 CN37 EL DORADO.xlsx</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>CN37</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="n">
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>BS37</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>BS37 - DORADO</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="inlineStr"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>SIN_MATCH_DB</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>Codigo 'CN37' no encontrado en DB.</t>
-        </is>
-      </c>
+      <c r="F51" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3951,7 +3967,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>CN35</t>
+          <t>BS35</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -4119,7 +4135,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>CN34</t>
+          <t>BS34</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -5517,7 +5533,7 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>CN26</t>
+          <t>BS26</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -6755,7 +6771,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
@@ -6765,7 +6781,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -6785,7 +6801,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -6879,10 +6895,10 @@
         <v>8</v>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -6895,13 +6911,13 @@
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
         <v>5</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Paso 6: agregar estado COT_DEBE_RECARGA para cotizaciones OCT mal emitidas
- Detecta automáticamente cuando una cotización de mes RECARGA coincide
  con precio MANTENIMIENTO (error confirmado por usuario para OCTUBRE)
- 5 locales marcados COT_DEBE_RECARGA (naranja), 43 INCONSISTENCIAS reales
- Fill naranja en Excel para distinguirlos de inconsistencias de precio

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/REVISION_COTIZACIONES_2026.xlsx
+++ b/REVISION_COTIZACIONES_2026.xlsx
@@ -35,7 +35,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B942"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,6 +102,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -6321,88 +6327,96 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="3" t="inlineStr">
+      <c r="A145" s="5" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B145" s="5" t="inlineStr">
         <is>
           <t>COTIZACION1217 M33 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C145" s="3" t="inlineStr">
+      <c r="C145" s="5" t="inlineStr">
         <is>
           <t>M33</t>
         </is>
       </c>
-      <c r="D145" s="3" t="inlineStr">
+      <c r="D145" s="5" t="inlineStr">
         <is>
           <t>M033 - CITY MALL</t>
         </is>
       </c>
-      <c r="E145" s="3" t="n">
+      <c r="E145" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F145" s="3" t="n">
+      <c r="F145" s="5" t="n">
         <v>63.8</v>
       </c>
-      <c r="G145" s="3" t="inlineStr">
+      <c r="G145" s="5" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H145" s="3" t="n">
+      <c r="H145" s="5" t="n">
         <v>56.11</v>
       </c>
-      <c r="I145" s="3" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J145" s="3" t="inlineStr"/>
+      <c r="I145" s="5" t="inlineStr">
+        <is>
+          <t>COT_DEBE_RECARGA</t>
+        </is>
+      </c>
+      <c r="J145" s="5" t="inlineStr">
+        <is>
+          <t>Cotización emitida como MANTENIMIENTO ($28.0=28.0), debe ser RECARGA ($63.8)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="3" t="inlineStr">
+      <c r="A146" s="5" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B146" s="3" t="inlineStr">
+      <c r="B146" s="5" t="inlineStr">
         <is>
           <t>COTIZACION1218 CJNC11 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C146" s="3" t="inlineStr">
+      <c r="C146" s="5" t="inlineStr">
         <is>
           <t>J11</t>
         </is>
       </c>
-      <c r="D146" s="3" t="inlineStr">
+      <c r="D146" s="5" t="inlineStr">
         <is>
           <t>J011 - CITY MALL</t>
         </is>
       </c>
-      <c r="E146" s="3" t="n">
+      <c r="E146" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F146" s="3" t="n">
+      <c r="F146" s="5" t="n">
         <v>63.8</v>
       </c>
-      <c r="G146" s="3" t="inlineStr">
+      <c r="G146" s="5" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H146" s="3" t="n">
+      <c r="H146" s="5" t="n">
         <v>56.11</v>
       </c>
-      <c r="I146" s="3" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J146" s="3" t="inlineStr"/>
+      <c r="I146" s="5" t="inlineStr">
+        <is>
+          <t>COT_DEBE_RECARGA</t>
+        </is>
+      </c>
+      <c r="J146" s="5" t="inlineStr">
+        <is>
+          <t>Cotización emitida como MANTENIMIENTO ($28.0=28.0), debe ser RECARGA ($63.8)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -6473,88 +6487,96 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="3" t="inlineStr">
+      <c r="A149" s="5" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B149" s="5" t="inlineStr">
         <is>
           <t>COTIZACION1221 M61 PORTETE.xlsx</t>
         </is>
       </c>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="C149" s="5" t="inlineStr">
         <is>
           <t>M61</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
+      <c r="D149" s="5" t="inlineStr">
         <is>
           <t>M061 - PORTETE</t>
         </is>
       </c>
-      <c r="E149" s="3" t="n">
+      <c r="E149" s="5" t="n">
         <v>64</v>
       </c>
-      <c r="F149" s="3" t="n">
+      <c r="F149" s="5" t="n">
         <v>152</v>
       </c>
-      <c r="G149" s="3" t="inlineStr">
+      <c r="G149" s="5" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H149" s="3" t="n">
+      <c r="H149" s="5" t="n">
         <v>57.89</v>
       </c>
-      <c r="I149" s="3" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J149" s="3" t="inlineStr"/>
+      <c r="I149" s="5" t="inlineStr">
+        <is>
+          <t>COT_DEBE_RECARGA</t>
+        </is>
+      </c>
+      <c r="J149" s="5" t="inlineStr">
+        <is>
+          <t>Cotización emitida como MANTENIMIENTO ($64.0=64.0), debe ser RECARGA ($152.0)</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" s="3" t="inlineStr">
+      <c r="A150" s="5" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B150" s="5" t="inlineStr">
         <is>
           <t>COTIZACION1222 KFCK109 CITY MALL PA.xlsx</t>
         </is>
       </c>
-      <c r="C150" s="3" t="inlineStr">
+      <c r="C150" s="5" t="inlineStr">
         <is>
           <t>K109</t>
         </is>
       </c>
-      <c r="D150" s="3" t="inlineStr">
+      <c r="D150" s="5" t="inlineStr">
         <is>
           <t>K109 - CITY MALL PA</t>
         </is>
       </c>
-      <c r="E150" s="3" t="n">
+      <c r="E150" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="F150" s="3" t="n">
+      <c r="F150" s="5" t="n">
         <v>72.8</v>
       </c>
-      <c r="G150" s="3" t="inlineStr">
+      <c r="G150" s="5" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H150" s="3" t="n">
+      <c r="H150" s="5" t="n">
         <v>56.04</v>
       </c>
-      <c r="I150" s="3" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J150" s="3" t="inlineStr"/>
+      <c r="I150" s="5" t="inlineStr">
+        <is>
+          <t>COT_DEBE_RECARGA</t>
+        </is>
+      </c>
+      <c r="J150" s="5" t="inlineStr">
+        <is>
+          <t>Cotización emitida como MANTENIMIENTO ($32.0=32.0), debe ser RECARGA ($72.8)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -6641,46 +6663,50 @@
       <c r="J152" s="3" t="inlineStr"/>
     </row>
     <row r="153">
-      <c r="A153" s="3" t="inlineStr">
+      <c r="A153" s="5" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr">
+      <c r="B153" s="5" t="inlineStr">
         <is>
           <t>COTIZACION1216 KFCK117 SEDALANA.xlsx</t>
         </is>
       </c>
-      <c r="C153" s="3" t="inlineStr">
+      <c r="C153" s="5" t="inlineStr">
         <is>
           <t>K117</t>
         </is>
       </c>
-      <c r="D153" s="3" t="inlineStr">
+      <c r="D153" s="5" t="inlineStr">
         <is>
           <t>K117 - 29 Y SEDALANA</t>
         </is>
       </c>
-      <c r="E153" s="3" t="n">
+      <c r="E153" s="5" t="n">
         <v>104</v>
       </c>
-      <c r="F153" s="3" t="n">
+      <c r="F153" s="5" t="n">
         <v>241.2</v>
       </c>
-      <c r="G153" s="3" t="inlineStr">
+      <c r="G153" s="5" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H153" s="3" t="n">
+      <c r="H153" s="5" t="n">
         <v>56.88</v>
       </c>
-      <c r="I153" s="3" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J153" s="3" t="inlineStr"/>
+      <c r="I153" s="5" t="inlineStr">
+        <is>
+          <t>COT_DEBE_RECARGA</t>
+        </is>
+      </c>
+      <c r="J153" s="5" t="inlineStr">
+        <is>
+          <t>Cotización emitida como MANTENIMIENTO ($104.0=104.0), debe ser RECARGA ($241.2)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -6735,7 +6761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6743,7 +6769,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>RESUMEN DE REVISION COTIZACIONES 2026</t>
         </is>
@@ -6777,279 +6803,324 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INCONSISTENCIAS (diferencia &gt; 1%)</t>
+          <t>INCONSISTENCIAS DE PRECIO (diferencia &gt; 1%)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SIN SUBTOTAL en cotizacion</t>
+          <t>COT_DEBE_RECARGA (emitida como MANT, debe ser RECARGA)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SIN MATCH en base de datos</t>
+          <t>SIN SUBTOTAL en cotizacion</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SIN VALOR en base de datos</t>
+          <t>SIN MATCH en base de datos (otras marcas)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>SIN VALOR en base de datos</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>ERRORES (descarga/parseo)</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>DETALLE POR MES</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MES</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>OTROS</t>
-        </is>
-      </c>
+          <t>DETALLE POR MES</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ENERO</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>24</v>
-      </c>
-      <c r="C13" t="n">
-        <v>19</v>
-      </c>
-      <c r="D13" t="n">
-        <v>5</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
+          <t>MES</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>INCONSISTENCIA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>COT_DEBE_RECARGA</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>OTROS</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FEBRERO</t>
+          <t>ENERO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C14" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MARZO</t>
+          <t>FEBRERO</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="n">
         <v>7</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
         <v>5</v>
-      </c>
-      <c r="E15" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABRIL</t>
+          <t>MARZO</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MAYO</t>
+          <t>ABRIL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>JUNIO</t>
+          <t>MAYO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C18" t="n">
         <v>6</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JULIO</t>
+          <t>JUNIO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AGOSTO</t>
+          <t>JULIO</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C20" t="n">
         <v>12</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SEPTIEMBRE</t>
+          <t>AGOSTO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="C21" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
         <v>3</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>SEPTIEMBRE</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B23" t="n">
         <v>11</v>
       </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>8</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Paso 6: corregir J20 viáticos $34→$68 y lógica AÑO_RECARGA para R3/R8/R10
- build_database.py: J20 GYE-LIBERTAD 136KM x2 = $68 (RETIRO+ENTREGA)
- build_database.py: COBRO_ANUAL total actualizado a $19,914.60
- revision_cotizaciones.py: cargar AÑO_RECARGA desde RESUMEN_LOCALES (row[9])
- revision_cotizaciones.py: comparar RECARGA para locales con AÑO_RECARGA=2026 en ENE-SEP
- Resultado: R3/R8/R10 ahora OK; 94 OK / 25 INCONSISTENCIAS / 5 COT_DEBE_RECARGA / 29 SIN_MATCH

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/REVISION_COTIZACIONES_2026.xlsx
+++ b/REVISION_COTIZACIONES_2026.xlsx
@@ -725,7 +725,7 @@
         <v>126.7</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H5" s="4" t="n">
-        <v>295.94</v>
+        <v>75.97</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
@@ -747,12 +747,12 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
+          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×MOVILIZACIÓN@$40</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>-2 ext en COT vs DB (2 vs 4) | ⚠ suma líneas COT=$81.80 ≠ subtotal=$126.70 | Extra en COT: +1×??(@$48) | Falta en COT: -1×50lbCO2, -1×10lbCO2, -1×10lbPQS</t>
+          <t>-3 ext en COT vs DB (2 vs 5) | ⚠ suma líneas COT=$81.80 ≠ subtotal=$126.70 | Extra en COT: +1×??(@$48) | Falta en COT: -1×50lbCO2, -1×10lbCO2, -1×10lbPQS, -1×MOVILIZACIÓN</t>
         </is>
       </c>
     </row>
@@ -1785,60 +1785,48 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1295 KFCK148 TERMINAL MACHALA.xlsx</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>K148</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>K148 - TERMINAL TERRESTRE MACHALA</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="2" t="n">
         <v>93.5</v>
       </c>
-      <c r="F28" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>146.05</v>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4 + 1×5lbPQS@$2 + 1×2.5glnK@$8</t>
-        </is>
-      </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbPQS@$2 + 1×2.5GLSTIPO K@$8 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$38.00 ≠ subtotal=$93.50 | Extra en COT: +1×2.5glnK(@$8) | Falta en COT: -1×2.5GLSTIPO K</t>
-        </is>
-      </c>
+      <c r="F28" s="2" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2205,228 +2193,180 @@
       <c r="L37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1308 JV75 PASEO SHOPPING MACHALA.xlsx</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>V75</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>V075 - PASEO SHOPPING MACHALA</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F38" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J38" s="5" t="inlineStr">
-        <is>
-          <t>2×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K38" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbCO2@$4 + 1×10lbCO2@$4</t>
-        </is>
-      </c>
-      <c r="L38" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$8.00 ≠ subtotal=$16.00 | Extra en COT: +2×10lbPQS(@$4) | Falta en COT: -2×10lbCO2</t>
-        </is>
-      </c>
+      <c r="F38" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1293 KFCK90 MACHALA CENTRO.xlsx</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>K90</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>K090 - MACHALA CENTRO</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="2" t="n">
         <v>111.5</v>
       </c>
-      <c r="F39" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="n">
-        <v>99.11</v>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 4×5lbCO2@$2 + 1×10lbPQS@$4 + 3×20lbPQS@$8</t>
-        </is>
-      </c>
-      <c r="K39" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×20lbPQS@$8 + 1×20lbPQS@$8 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$56.00 ≠ subtotal=$111.50</t>
-        </is>
-      </c>
+      <c r="F39" s="2" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1294 KFCK91PASEO SHOPP MACHALA.xlsx</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>K91</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>K091 - MACHALA RIO CENTRO</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" s="2" t="n">
         <v>87.5</v>
       </c>
-      <c r="F40" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>173.44</v>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×2.5glnK@$8 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×2.5GLSTIPO K@$8 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$32.00 ≠ subtotal=$87.50 | Extra en COT: +1×2.5glnK(@$8) | Falta en COT: -1×2.5GLSTIPO K</t>
-        </is>
-      </c>
+      <c r="F40" s="2" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1292 KFCK65 MILAGRO.xlsx</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>K65</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>K065 - MILAGRO</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="F41" s="4" t="n">
-        <v>36</v>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>69.44</v>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 3×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K41" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbCO2@$4</t>
-        </is>
-      </c>
-      <c r="L41" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$36.00 ≠ subtotal=$61.00</t>
-        </is>
-      </c>
+      <c r="F41" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2473,60 +2413,48 @@
       <c r="L42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1309 JV79 MILAGRO.xlsx</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>V79</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>V079 - MILAGRO</t>
         </is>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F43" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>2×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K43" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$8.00 ≠ subtotal=$16.00</t>
-        </is>
-      </c>
+      <c r="F43" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr"/>
+      <c r="K43" s="3" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -3429,60 +3357,48 @@
       <c r="L63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>ABRIL</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1401 KFCK82 PLAYAS.xlsx</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>K82</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>K082 - SHOPPING PLAYAS</t>
         </is>
       </c>
-      <c r="E64" s="4" t="n">
+      <c r="E64" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="F64" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="n">
-        <v>137.5</v>
-      </c>
-      <c r="I64" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J64" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 2×10lbPQS@$4 + 2×5lbPQS@$2</t>
-        </is>
-      </c>
-      <c r="K64" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×5lbPQS@$2 + 1×5lbPQS@$2</t>
-        </is>
-      </c>
-      <c r="L64" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$32.00 ≠ subtotal=$76.00</t>
-        </is>
-      </c>
+      <c r="F64" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr"/>
+      <c r="L64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3609,15 +3525,15 @@
         <v>33.8</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>42</v>
+        <v>97.7</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>RECARGA</t>
         </is>
       </c>
       <c r="H67" s="4" t="n">
-        <v>19.52</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
@@ -3631,7 +3547,7 @@
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×20lbPQS@$8</t>
+          <t>1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×20lbPQS@$20</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
@@ -4069,172 +3985,136 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="inlineStr">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1463 R010 ORELLANA.xlsx</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>R010 - FRANCISCO DE ORELLANA</t>
         </is>
       </c>
-      <c r="E78" s="4" t="n">
+      <c r="E78" s="2" t="n">
         <v>418.7</v>
       </c>
-      <c r="F78" s="4" t="n">
-        <v>102</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="n">
-        <v>310.49</v>
-      </c>
-      <c r="I78" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J78" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$68 + 2×10lbCO2@$9 + 4×5lbCO2@$4 + 1×20lbPQS@$20 + 10×10lbPQS@$10 + 2×2.5glnK@$99</t>
-        </is>
-      </c>
-      <c r="K78" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×10lbCO2@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8 + 1×2.5GLSTIPO K@$8</t>
-        </is>
-      </c>
-      <c r="L78" s="5" t="inlineStr">
-        <is>
-          <t>+2 ext en COT vs DB (20 vs 18) | Extra en COT: +1×10lbCO2(@$9), +1×10lbPQS(@$10), +2×2.5glnK(@$99) | Falta en COT: -2×2.5GLSTIPO K</t>
-        </is>
-      </c>
+      <c r="F78" s="2" t="n">
+        <v>418.7</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>RECARGA</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr"/>
+      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1462 R008 MALL DEL SOL.xlsx</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>R008 - MALL DEL SOL</t>
         </is>
       </c>
-      <c r="E79" s="4" t="n">
+      <c r="E79" s="2" t="n">
         <v>232.5</v>
       </c>
-      <c r="F79" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="n">
-        <v>252.27</v>
-      </c>
-      <c r="I79" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J79" s="5" t="inlineStr">
-        <is>
-          <t>2×50lbCO2@$45 + 1×5lbCO2@$4 + 4×10lbPQS@$10 + 1×2.5glnK@$99</t>
-        </is>
-      </c>
-      <c r="K79" s="5" t="inlineStr">
-        <is>
-          <t>1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×50lbCO2@$20 + 1×50lbCO2@$20 + 1×2.5GLSTIPO K@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L79" s="5" t="inlineStr">
-        <is>
-          <t>Extra en COT: +1×2.5glnK(@$99) | Falta en COT: -1×2.5GLSTIPO K</t>
-        </is>
-      </c>
+      <c r="F79" s="2" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>RECARGA</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1461 R003 CENTRO.xlsx</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>R003 - 9 DE OCTUBRE</t>
         </is>
       </c>
-      <c r="E80" s="4" t="n">
+      <c r="E80" s="2" t="n">
         <v>192</v>
       </c>
-      <c r="F80" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="n">
-        <v>300</v>
-      </c>
-      <c r="I80" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J80" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$45 + 2×5lbCO2@$4 + 4×10lbPQS@$10 + 1×2.5glnK@$99</t>
-        </is>
-      </c>
-      <c r="K80" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×50lbCO2@$20 + 1×2.5GLSTIPO K@$8</t>
-        </is>
-      </c>
-      <c r="L80" s="5" t="inlineStr">
-        <is>
-          <t>Extra en COT: +1×2.5glnK(@$99) | Falta en COT: -1×2.5GLSTIPO K</t>
-        </is>
-      </c>
+      <c r="F80" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>RECARGA</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr"/>
+      <c r="K80" s="3" t="inlineStr"/>
+      <c r="L80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -4317,15 +4197,15 @@
         <v>90</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>102</v>
+        <v>418.7</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
+          <t>RECARGA</t>
         </is>
       </c>
       <c r="H82" s="4" t="n">
-        <v>11.76</v>
+        <v>78.5</v>
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
@@ -4339,12 +4219,12 @@
       </c>
       <c r="K82" s="5" t="inlineStr">
         <is>
-          <t>1×75lbCO2@$30 + 1×10lbCO2@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8 + 1×2.5GLSTIPO K@$8</t>
+          <t>1×75lbCO2@$68 + 1×10lbCO2@$9 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×20lbPQS@$20 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×2.5GLSTIPO K@$99 + 1×2.5GLSTIPO K@$99 + 1×MOVILIZACIÓN@$19</t>
         </is>
       </c>
       <c r="L82" s="5" t="inlineStr">
         <is>
-          <t>-18 ext en COT vs DB (0 vs 18) | ⚠ suma líneas COT=$0.00 ≠ subtotal=$90.00 | Falta en COT: -1×75lbCO2, -1×10lbCO2, -4×5lbCO2, -1×20lbPQS, -9×10lbPQS, -2×2.5GLSTIPO K</t>
+          <t>-19 ext en COT vs DB (0 vs 19) | ⚠ suma líneas COT=$0.00 ≠ subtotal=$90.00 | Falta en COT: -1×75lbCO2, -1×10lbCO2, -4×5lbCO2, -1×20lbPQS, -9×10lbPQS, -2×2.5GLSTIPO K, -1×MOVILIZACIÓN</t>
         </is>
       </c>
     </row>
@@ -4869,7 +4749,7 @@
         <v>76</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
@@ -4877,7 +4757,7 @@
         </is>
       </c>
       <c r="H94" s="4" t="n">
-        <v>137.5</v>
+        <v>5.56</v>
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
@@ -4891,12 +4771,12 @@
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
+          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×MOVILIZACIÓN@$40</t>
         </is>
       </c>
       <c r="L94" s="5" t="inlineStr">
         <is>
-          <t>+1 ext en COT vs DB (5 vs 4) | ⚠ suma líneas COT=$36.00 ≠ subtotal=$76.00 | Extra en COT: +1×10lbCO2(@$4)</t>
+          <t>⚠ suma líneas COT=$36.00 ≠ subtotal=$76.00 | Extra en COT: +1×10lbCO2(@$4) | Falta en COT: -1×MOVILIZACIÓN</t>
         </is>
       </c>
     </row>
@@ -5069,60 +4949,48 @@
       <c r="L98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="inlineStr">
+      <c r="A99" s="2" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B99" s="4" t="inlineStr">
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1569 KFCK93 QUEVEDO CENTRO.xlsx</t>
         </is>
       </c>
-      <c r="C99" s="4" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>K93</t>
         </is>
       </c>
-      <c r="D99" s="4" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>K093 - QUEVEDO</t>
         </is>
       </c>
-      <c r="E99" s="4" t="n">
+      <c r="E99" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="F99" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="G99" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H99" s="4" t="n">
-        <v>79.55</v>
-      </c>
-      <c r="I99" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J99" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 2×10lbPQS@$4 + 2×20lbPQS@$8</t>
-        </is>
-      </c>
-      <c r="K99" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×20lbPQS@$8 + 1×20lbPQS@$8</t>
-        </is>
-      </c>
-      <c r="L99" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$44.00 ≠ subtotal=$79.00</t>
-        </is>
-      </c>
+      <c r="F99" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr"/>
+      <c r="K99" s="3" t="inlineStr"/>
+      <c r="L99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5205,60 +5073,48 @@
       <c r="L101" s="7" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="inlineStr">
+      <c r="A102" s="2" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B102" s="4" t="inlineStr">
+      <c r="B102" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1564 CJNC20 LIBERTAD.xlsx</t>
         </is>
       </c>
-      <c r="C102" s="4" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>J20</t>
         </is>
       </c>
-      <c r="D102" s="4" t="inlineStr">
+      <c r="D102" s="2" t="inlineStr">
         <is>
           <t>J020 - CAJUN PENINSULA</t>
         </is>
       </c>
-      <c r="E102" s="4" t="n">
+      <c r="E102" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="F102" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="G102" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H102" s="4" t="n">
-        <v>178.95</v>
-      </c>
-      <c r="I102" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J102" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K102" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L102" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$38.00 ≠ subtotal=$106.00</t>
-        </is>
-      </c>
+      <c r="F102" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr"/>
+      <c r="K102" s="3" t="inlineStr"/>
+      <c r="L102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
@@ -5341,60 +5197,48 @@
       <c r="L104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="4" t="inlineStr">
+      <c r="A105" s="2" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B105" s="4" t="inlineStr">
+      <c r="B105" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1565 KFCK78 DAULE.xlsx</t>
         </is>
       </c>
-      <c r="C105" s="4" t="inlineStr">
+      <c r="C105" s="2" t="inlineStr">
         <is>
           <t>K78</t>
         </is>
       </c>
-      <c r="D105" s="4" t="inlineStr">
+      <c r="D105" s="2" t="inlineStr">
         <is>
           <t>K078 - SHOPPING DAULE</t>
         </is>
       </c>
-      <c r="E105" s="4" t="n">
+      <c r="E105" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="F105" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="G105" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H105" s="4" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="I105" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J105" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 2×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K105" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L105" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$30.00 ≠ subtotal=$55.00</t>
-        </is>
-      </c>
+      <c r="F105" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr"/>
+      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5821,60 +5665,48 @@
       <c r="L115" s="7" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" s="4" t="inlineStr">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B116" s="4" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1573 KFCK149 VENTANAS.xlsx</t>
         </is>
       </c>
-      <c r="C116" s="4" t="inlineStr">
+      <c r="C116" s="2" t="inlineStr">
         <is>
           <t>K149</t>
         </is>
       </c>
-      <c r="D116" s="4" t="inlineStr">
+      <c r="D116" s="2" t="inlineStr">
         <is>
           <t>K149 - PETROCOMERIAL VENTANAS</t>
         </is>
       </c>
-      <c r="E116" s="4" t="n">
+      <c r="E116" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="F116" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G116" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H116" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="I116" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J116" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 2×10lbPQS@$4 + 1×2.5glnK@$8</t>
-        </is>
-      </c>
-      <c r="K116" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L116" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$50.00 ≠ subtotal=$85.00 | Extra en COT: +1×2.5glnK(@$8) | Falta en COT: -1×2.5GLSTIPO K</t>
-        </is>
-      </c>
+      <c r="F116" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr"/>
+      <c r="K116" s="3" t="inlineStr"/>
+      <c r="L116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -5989,60 +5821,48 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="4" t="inlineStr">
+      <c r="A119" s="2" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1570 KFCK106 SHOPPING QUEVEDO.xlsx</t>
         </is>
       </c>
-      <c r="C119" s="4" t="inlineStr">
+      <c r="C119" s="2" t="inlineStr">
         <is>
           <t>K106</t>
         </is>
       </c>
-      <c r="D119" s="4" t="inlineStr">
+      <c r="D119" s="2" t="inlineStr">
         <is>
           <t>K106 - SHOPPING QUEVEDO</t>
         </is>
       </c>
-      <c r="E119" s="4" t="n">
+      <c r="E119" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="F119" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="G119" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H119" s="4" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="I119" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J119" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 2×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K119" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2</t>
-        </is>
-      </c>
-      <c r="L119" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$42.00 ≠ subtotal=$77.00</t>
-        </is>
-      </c>
+      <c r="F119" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr"/>
+      <c r="K119" s="3" t="inlineStr"/>
+      <c r="L119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
@@ -6081,116 +5901,92 @@
       <c r="L120" s="7" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" s="4" t="inlineStr">
+      <c r="A121" s="2" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B121" s="4" t="inlineStr">
+      <c r="B121" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1572 M32 SHOPPING QUEVEDO.xlsx</t>
         </is>
       </c>
-      <c r="C121" s="4" t="inlineStr">
+      <c r="C121" s="2" t="inlineStr">
         <is>
           <t>M32</t>
         </is>
       </c>
-      <c r="D121" s="4" t="inlineStr">
+      <c r="D121" s="2" t="inlineStr">
         <is>
           <t>M032 - SHOPPING QUEVEDO</t>
         </is>
       </c>
-      <c r="E121" s="4" t="n">
+      <c r="E121" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="F121" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="G121" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H121" s="4" t="n">
-        <v>92.11</v>
-      </c>
-      <c r="I121" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J121" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K121" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L121" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$38.00 ≠ subtotal=$73.00</t>
-        </is>
-      </c>
+      <c r="F121" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="inlineStr"/>
+      <c r="L121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="4" t="inlineStr">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1606 M39 BABAHOYO.xlsx</t>
         </is>
       </c>
-      <c r="C122" s="4" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>M39</t>
         </is>
       </c>
-      <c r="D122" s="4" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>M039 - PASEO SHOPPING BABAHOYO</t>
         </is>
       </c>
-      <c r="E122" s="4" t="n">
+      <c r="E122" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="F122" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G122" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H122" s="4" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="I122" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J122" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K122" s="5" t="inlineStr">
-        <is>
-          <t>1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×50lbCO2@$20 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L122" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$28.00 ≠ subtotal=$52.00</t>
-        </is>
-      </c>
+      <c r="F122" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J122" s="3" t="inlineStr"/>
+      <c r="K122" s="3" t="inlineStr"/>
+      <c r="L122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
@@ -6229,60 +6025,48 @@
       <c r="L123" s="7" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="4" t="inlineStr">
+      <c r="A124" s="2" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="B124" s="4" t="inlineStr">
+      <c r="B124" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1603 KFCK53 SHOPPING BABAHOYO.xlsx</t>
         </is>
       </c>
-      <c r="C124" s="4" t="inlineStr">
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>K53</t>
         </is>
       </c>
-      <c r="D124" s="4" t="inlineStr">
+      <c r="D124" s="2" t="inlineStr">
         <is>
           <t>K053 - PASEO SHOPPING BABAHOYO</t>
         </is>
       </c>
-      <c r="E124" s="4" t="n">
+      <c r="E124" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="F124" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G124" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H124" s="4" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="I124" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J124" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K124" s="5" t="inlineStr">
-        <is>
-          <t>1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×50lbCO2@$20 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L124" s="5" t="inlineStr">
-        <is>
-          <t>⚠ suma líneas COT=$28.00 ≠ subtotal=$52.00</t>
-        </is>
-      </c>
+      <c r="F124" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J124" s="3" t="inlineStr"/>
+      <c r="K124" s="3" t="inlineStr"/>
+      <c r="L124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -7691,7 +7475,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5">
@@ -7701,7 +7485,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -7809,10 +7593,10 @@
         <v>20</v>
       </c>
       <c r="C12" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -7859,10 +7643,10 @@
         <v>8</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -7884,10 +7668,10 @@
         <v>15</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -7934,10 +7718,10 @@
         <v>26</v>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -7959,10 +7743,10 @@
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Correcciones manuales de inventario por local (revisión cotizaciones 2026)
- build_database.py: capa EXTINTOR_OVERRIDE con inventario confirmado de 22 locales
- Eliminado K124 (Gran Aki Loja - ya no se atiende) → 197 locales
- K79 movido a JUNIO, K88 movido a OCTUBRE (cotizaciones de enero/abril eran ventas)
- R004: AÑO recarga 2025/próxima 2028 (mantenimiento en mayo 2026)
- R010: inventario completo (recarga+mantt mayo 2026)
- revision_cotizaciones.py: estado VENTA para cotizaciones que no son mantto/recarga
- Inconsistencias 25→14, OK 94→102, Cobro anual $20,134.20

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/REVISION_COTIZACIONES_2026.xlsx
+++ b/REVISION_COTIZACIONES_2026.xlsx
@@ -35,7 +35,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,6 +126,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -733,20 +744,16 @@
       <c r="E5" s="4" t="n">
         <v>126.7</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>72</v>
-      </c>
+      <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>75.97</v>
-      </c>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>INCONSISTENCIA</t>
+          <t>VENTA</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -754,19 +761,15 @@
           <t>1×??@$48 + 1×10lbPQS@$34  [+MOVIL:$40.00 — MOVILIZACION (GYE - BABAHOYO)]</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4  [+MOVIL:$40.00 — GYE-BABAHOYO 75KM]</t>
-        </is>
-      </c>
+      <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Extintores COT=$81.80 vs DB=$32.00 (neto +$49.80) | Cantidad: 2 ext en COT vs 4 en DB | COT tiene +1×?? que no está en DB (precio $48/ext) | DB tiene +1×50lbCO2 que no aparece en COT ($20/ext) | DB tiene +1×10lbCO2 que no aparece en COT ($4/ext) | DB tiene +1×10lbPQS que no aparece en COT ($4/ext)</t>
+          <t>Cotización por venta de extintores / servicio, no mantenimiento</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>¿AGREGAR 1×?? a BD? ($48/ext) | ¿RETIRAR 1×50lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×10lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×10lbPQS de BD? (o verificar si fue omitido en COT)</t>
+          <t>Informativo — no afecta la base de datos</t>
         </is>
       </c>
     </row>
@@ -906,126 +909,94 @@
       <c r="M8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ENERO</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1262 KFCK25 MOBIL DURAN.xlsx</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>K25</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>K025 - MOBIL DURAN</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>9.52</v>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×10lbCO2@$4 + 3×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbCO2@$4 + 1×75lbCO2@$30 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$46.00 vs DB=$42.00 (neto +$4.00) | Cantidad: 5 ext en COT vs 4 en DB | COT tiene +1×10lbPQS que no está en DB (precio $4/ext)</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbPQS a BD? ($4/ext)</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ENERO</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1273 KFCK154 PASCUALES.xlsx</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>K154</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>K154 - PASCUALES</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 3×5lbCO2@$2 + 1×20lbPQS@$8 + 3×10lbPQS@$4 + 1×2.5glnK@$8</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$54.00 vs DB=$52.00 (neto +$2.00) | Cantidad: 9 ext en COT vs 8 en DB | COT tiene +1×5lbCO2 que no está en DB (precio $2/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×5lbCO2 a BD? ($2/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1253,61 +1224,61 @@
       <c r="M15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>ENERO</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1267 KFCK76 PARQUE CENTENARIO.xlsx</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>K76</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>K076 - PARQUE CENTENARIO</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="n">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 3×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
         <is>
           <t>Extintores COT=$36.00 vs DB=$40.00 (neto $-4.00) | Cantidad: 6 ext en COT vs 7 en DB | DB tiene +1×10lbPQS que no aparece en COT ($4/ext)</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>¿RETIRAR 1×10lbPQS de BD? (o verificar si fue omitido en COT)</t>
         </is>
@@ -1584,61 +1555,61 @@
       <c r="M22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>ENERO</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1271 KFCK105 RIOCENTRO NORTE.xlsx</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>K105</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>K105 - HIPER MARKET</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="n">
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="n">
         <v>4.55</v>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>1×75lbCO2@$30 + 1×5lbCO2@$4 + 1×20lbPQS@$8 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>1×75lbCO2@$30 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="L23" s="7" t="inlineStr">
         <is>
           <t>Extintores COT=$46.00 vs DB=$44.00 (neto +$2.00) | 1×5lbCO2: precio COT=$4 vs DB=$2/ext</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M23" s="7" t="inlineStr">
         <is>
           <t>¿Actualizar precio 5lbCO2 en BD: $2→$4/ext?</t>
         </is>
@@ -1780,65 +1751,49 @@
       <c r="M26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1291 KFCK45 BOYACA.xlsx</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>K45</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>K045 - BOYACA</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="F27" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 3×20lbPQS@$8 + 6×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×20lbPQS@$8 + 1×20lbPQS@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$70.00 vs DB=$66.00 (neto +$4.00) | Cantidad: 11 ext en COT vs 10 en DB | COT tiene +1×10lbPQS que no está en DB (precio $4/ext)</t>
-        </is>
-      </c>
-      <c r="M27" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbPQS a BD? ($4/ext)</t>
-        </is>
-      </c>
+      <c r="F27" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1976,115 +1931,115 @@
       <c r="M30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1301 ESPE06 MALL DEL SOL.xlsx</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>ESPE6</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr"/>
-      <c r="E31" s="6" t="n">
+      <c r="D31" s="8" t="inlineStr"/>
+      <c r="E31" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="inlineStr"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="inlineStr"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="J31" s="9" t="inlineStr">
         <is>
           <t>1×10lbPQS@$4 + 1×5lbCO2@$2</t>
         </is>
       </c>
-      <c r="K31" s="7" t="inlineStr"/>
-      <c r="L31" s="7" t="inlineStr"/>
-      <c r="M31" s="7" t="inlineStr"/>
+      <c r="K31" s="9" t="inlineStr"/>
+      <c r="L31" s="9" t="inlineStr"/>
+      <c r="M31" s="9" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1302 ESPE10 SAN MARINO.xlsx</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>ESPE10</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr"/>
-      <c r="E32" s="6" t="n">
+      <c r="D32" s="8" t="inlineStr"/>
+      <c r="E32" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="inlineStr">
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="inlineStr"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="J32" s="9" t="inlineStr">
         <is>
           <t>2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K32" s="7" t="inlineStr"/>
-      <c r="L32" s="7" t="inlineStr"/>
-      <c r="M32" s="7" t="inlineStr"/>
+      <c r="K32" s="9" t="inlineStr"/>
+      <c r="L32" s="9" t="inlineStr"/>
+      <c r="M32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1303 ESPE26 RIOC PUNTILLA.xlsx</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>ESPE26</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr"/>
-      <c r="E33" s="6" t="n">
+      <c r="D33" s="8" t="inlineStr"/>
+      <c r="E33" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="inlineStr"/>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="inlineStr"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr">
+      <c r="J33" s="9" t="inlineStr">
         <is>
           <t>1×10lbPQS@$4 + 1×5lbPQS@$2 + 1×5lbCO2@$2</t>
         </is>
       </c>
-      <c r="K33" s="7" t="inlineStr"/>
-      <c r="L33" s="7" t="inlineStr"/>
-      <c r="M33" s="7" t="inlineStr"/>
+      <c r="K33" s="9" t="inlineStr"/>
+      <c r="L33" s="9" t="inlineStr"/>
+      <c r="M33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2222,41 +2177,41 @@
       <c r="M36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1307 ILCI02 RIOC. CEIBOS.xlsx</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>ILCI2</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr"/>
-      <c r="E37" s="6" t="n">
+      <c r="D37" s="8" t="inlineStr"/>
+      <c r="E37" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="inlineStr"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="6" t="inlineStr">
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="inlineStr"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
+      <c r="J37" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K37" s="7" t="inlineStr"/>
-      <c r="L37" s="7" t="inlineStr"/>
-      <c r="M37" s="7" t="inlineStr"/>
+      <c r="K37" s="9" t="inlineStr"/>
+      <c r="L37" s="9" t="inlineStr"/>
+      <c r="M37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2529,41 +2484,41 @@
       <c r="M43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>FEBRERO</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1296 AMCA37 EL DORADO.xlsx</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
         <is>
           <t>AMCA37</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr"/>
-      <c r="E44" s="6" t="n">
+      <c r="D44" s="8" t="inlineStr"/>
+      <c r="E44" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="6" t="inlineStr"/>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="6" t="inlineStr">
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="inlineStr"/>
+      <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J44" s="7" t="inlineStr">
+      <c r="J44" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×10lbCO2@$4 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K44" s="7" t="inlineStr"/>
-      <c r="L44" s="7" t="inlineStr"/>
-      <c r="M44" s="7" t="inlineStr"/>
+      <c r="K44" s="9" t="inlineStr"/>
+      <c r="L44" s="9" t="inlineStr"/>
+      <c r="M44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2611,41 +2566,41 @@
       <c r="M45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1352 GUSG49 DURAN.xlsx</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>GUSG49</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr"/>
-      <c r="E46" s="6" t="n">
+      <c r="D46" s="8" t="inlineStr"/>
+      <c r="E46" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="inlineStr"/>
-      <c r="H46" s="6" t="n"/>
-      <c r="I46" s="6" t="inlineStr">
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="inlineStr"/>
+      <c r="H46" s="8" t="n"/>
+      <c r="I46" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J46" s="7" t="inlineStr">
+      <c r="J46" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K46" s="7" t="inlineStr"/>
-      <c r="L46" s="7" t="inlineStr"/>
-      <c r="M46" s="7" t="inlineStr"/>
+      <c r="K46" s="9" t="inlineStr"/>
+      <c r="L46" s="9" t="inlineStr"/>
+      <c r="M46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2738,102 +2693,86 @@
       <c r="M48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1357 ILCI05 SAN MARINO.xlsx</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>ILCI5</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr"/>
-      <c r="E49" s="6" t="n">
+      <c r="D49" s="8" t="inlineStr"/>
+      <c r="E49" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="6" t="inlineStr"/>
-      <c r="H49" s="6" t="n"/>
-      <c r="I49" s="6" t="inlineStr">
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="8" t="inlineStr"/>
+      <c r="H49" s="8" t="n"/>
+      <c r="I49" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J49" s="7" t="inlineStr">
+      <c r="J49" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×2.5glnK@$8</t>
         </is>
       </c>
-      <c r="K49" s="7" t="inlineStr"/>
-      <c r="L49" s="7" t="inlineStr"/>
-      <c r="M49" s="7" t="inlineStr"/>
+      <c r="K49" s="9" t="inlineStr"/>
+      <c r="L49" s="9" t="inlineStr"/>
+      <c r="M49" s="9" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1358 KFCK75 MOBIL KENNEDY.xlsx</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>K75</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>K075 - MOBIL KENNEDY</t>
         </is>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="F50" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J50" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 2×10lbPQS@$4 + 1×20lbPQS@$8</t>
-        </is>
-      </c>
-      <c r="K50" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L50" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$40.00 vs DB=$32.00 (neto +$8.00) | Cantidad: 5 ext en COT vs 4 en DB | COT tiene +1×20lbPQS que no está en DB (precio $8/ext)</t>
-        </is>
-      </c>
-      <c r="M50" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×20lbPQS a BD? ($8/ext)</t>
-        </is>
-      </c>
+      <c r="F50" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3016,246 +2955,214 @@
       <c r="M54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1350 KFCK94 PASEO SHOPPING DURAN.xlsx</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>K94</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>K094 - OUTLET DURAN</t>
         </is>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E55" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F55" s="4" t="n">
+      <c r="F55" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="n">
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="n">
         <v>6.25</v>
       </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="I55" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J55" s="5" t="inlineStr">
+      <c r="J55" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K55" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×10lbCO2@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2</t>
-        </is>
-      </c>
-      <c r="L55" s="5" t="inlineStr">
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4</t>
+        </is>
+      </c>
+      <c r="L55" s="7" t="inlineStr">
         <is>
           <t>Extintores COT=$30.00 vs DB=$32.00 (neto $-2.00) | Cantidad: 4 ext en COT vs 5 en DB | DB tiene +1×5lbCO2 que no aparece en COT ($2/ext)</t>
         </is>
       </c>
-      <c r="M55" s="5" t="inlineStr">
+      <c r="M55" s="7" t="inlineStr">
         <is>
           <t>¿RETIRAR 1×5lbCO2 de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>MARZO</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1353 M11 MALL DEL SUR.xlsx</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>M11</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>M011 - MALL SUR</t>
         </is>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E56" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="F56" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>26.32</v>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
+      <c r="F56" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr"/>
+      <c r="K56" s="3" t="inlineStr"/>
+      <c r="L56" s="3" t="inlineStr"/>
+      <c r="M56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>MARZO</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>COTIZACION1351 KFCK145 AKI SAN EDUARDO.xlsx</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>K145</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>K145 - SUPER AKI SAN EDUARDO</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr"/>
+      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr"/>
+      <c r="M57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>MARZO</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>COTIZACION1354 M37 CENTRO.xlsx</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>M37</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>M037 - 9 DE OCTUBRE</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>20.83</v>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 2×10lbPQS@$4 + 1×5lbCO2@$2 + 1×2.5glnK@$8</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L56" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$48.00 vs DB=$38.00 (neto +$10.00) | Cantidad: 5 ext en COT vs 3 en DB | COT tiene +1×5lbCO2 que no está en DB (precio $2/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext)</t>
-        </is>
-      </c>
-      <c r="M56" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×5lbCO2 a BD? ($2/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>COTIZACION1351 KFCK145 AKI SAN EDUARDO.xlsx</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>K145</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>K145 - SUPER AKI SAN EDUARDO</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F57" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="n">
-        <v>19.05</v>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 3×5lbCO2@$2 + 2×10lbPQS@$4 + 1×2.5glnK@$8 + 1×20lbPQS@$8</t>
-        </is>
-      </c>
-      <c r="K57" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×50lbCO2@$20</t>
-        </is>
-      </c>
-      <c r="L57" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$50.00 vs DB=$42.00 (neto +$8.00) | Cantidad: 8 ext en COT vs 7 en DB | COT tiene +1×20lbPQS que no está en DB (precio $8/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M57" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×20lbPQS a BD? ($8/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>COTIZACION1354 M37 CENTRO.xlsx</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>M37</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>M037 - 9 DE OCTUBRE</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="F58" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="n">
-        <v>20.83</v>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J58" s="5" t="inlineStr">
+      <c r="J58" s="7" t="inlineStr">
         <is>
           <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 6×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K58" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L58" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$58.00 vs DB=$48.00 (neto +$10.00) | COT tiene +1×75lbCO2 que no está en DB (precio $30/ext) | DB tiene +1×50lbCO2 que no aparece en COT ($20/ext)</t>
-        </is>
-      </c>
-      <c r="M58" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×75lbCO2 a BD? ($30/ext) | ¿RETIRAR 1×50lbCO2 de BD? (o verificar si fue omitido en COT)</t>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$58.00 vs DB=$48.00 (neto +$10.00) | Cantidad: 9 ext en COT vs 8 en DB | COT tiene +1×75lbCO2 que no está en DB (precio $30/ext) | COT tiene +2×10lbPQS que no está en DB (precio $4/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext) | DB tiene +1×50lbCO2 que no aparece en COT ($20/ext)</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>¿AGREGAR 1×75lbCO2 a BD? ($30/ext) | ¿AGREGAR 2×10lbPQS a BD? ($4/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×50lbCO2 de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
@@ -3305,41 +3212,41 @@
       <c r="M59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>ABRIL</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1404 ILCI12 TERMINAL.xlsx</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="8" t="inlineStr">
         <is>
           <t>ILCI12</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr"/>
-      <c r="E60" s="6" t="n">
+      <c r="D60" s="8" t="inlineStr"/>
+      <c r="E60" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="6" t="n"/>
-      <c r="I60" s="6" t="inlineStr">
+      <c r="F60" s="8" t="n"/>
+      <c r="G60" s="8" t="inlineStr"/>
+      <c r="H60" s="8" t="n"/>
+      <c r="I60" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J60" s="7" t="inlineStr">
+      <c r="J60" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×2.5glnK@$8</t>
         </is>
       </c>
-      <c r="K60" s="7" t="inlineStr"/>
-      <c r="L60" s="7" t="inlineStr"/>
-      <c r="M60" s="7" t="inlineStr"/>
+      <c r="K60" s="9" t="inlineStr"/>
+      <c r="L60" s="9" t="inlineStr"/>
+      <c r="M60" s="9" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3387,41 +3294,41 @@
       <c r="M61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>ABRIL</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1403 GUSG45 TUNGURAHUA.xlsx</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>GUSG45</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr"/>
-      <c r="E62" s="6" t="n">
+      <c r="D62" s="8" t="inlineStr"/>
+      <c r="E62" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="inlineStr"/>
-      <c r="H62" s="6" t="n"/>
-      <c r="I62" s="6" t="inlineStr">
+      <c r="F62" s="8" t="n"/>
+      <c r="G62" s="8" t="inlineStr"/>
+      <c r="H62" s="8" t="n"/>
+      <c r="I62" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J62" s="7" t="inlineStr">
+      <c r="J62" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 3×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K62" s="7" t="inlineStr"/>
-      <c r="L62" s="7" t="inlineStr"/>
-      <c r="M62" s="7" t="inlineStr"/>
+      <c r="K62" s="9" t="inlineStr"/>
+      <c r="L62" s="9" t="inlineStr"/>
+      <c r="M62" s="9" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3559,65 +3466,41 @@
       <c r="M65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>ABRIL</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1400 KFCK124 GRAN AKI LOJA.xlsx</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C66" s="8" t="inlineStr">
         <is>
           <t>K124</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>K124 - GRAN AKI</t>
-        </is>
-      </c>
-      <c r="E66" s="4" t="n">
+      <c r="D66" s="8" t="inlineStr"/>
+      <c r="E66" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F66" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G66" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H66" s="4" t="n">
-        <v>28.57</v>
-      </c>
-      <c r="I66" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J66" s="5" t="inlineStr">
+      <c r="F66" s="8" t="n"/>
+      <c r="G66" s="8" t="inlineStr"/>
+      <c r="H66" s="8" t="n"/>
+      <c r="I66" s="8" t="inlineStr">
+        <is>
+          <t>SIN_MATCH_DB</t>
+        </is>
+      </c>
+      <c r="J66" s="9" t="inlineStr">
         <is>
           <t>3×10lbCO2@$4 + 1×20lbPQS@$8</t>
         </is>
       </c>
-      <c r="K66" s="5" t="inlineStr">
-        <is>
-          <t>1×10lbCO2@$4 + 1×10lbCO2@$4 + 1×10lbCO2@$4 + 1×20lbPQS@$8 + 1×2.5GLSTIPO K@$8</t>
-        </is>
-      </c>
-      <c r="L66" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$20.00 vs DB=$28.00 (neto $-8.00) | Cantidad: 4 ext en COT vs 5 en DB | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M66" s="5" t="inlineStr">
-        <is>
-          <t>¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
-        </is>
-      </c>
+      <c r="K66" s="9" t="inlineStr"/>
+      <c r="L66" s="9" t="inlineStr"/>
+      <c r="M66" s="9" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -3643,20 +3526,16 @@
       <c r="E67" s="4" t="n">
         <v>33.8</v>
       </c>
-      <c r="F67" s="4" t="n">
-        <v>97.7</v>
-      </c>
+      <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>RECARGA</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="n">
-        <v>65.40000000000001</v>
-      </c>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>INCONSISTENCIA</t>
+          <t>VENTA</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
@@ -3664,19 +3543,15 @@
           <t>1×10lbPQS@$34</t>
         </is>
       </c>
-      <c r="K67" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×20lbPQS@$20</t>
-        </is>
-      </c>
+      <c r="K67" s="5" t="inlineStr"/>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>Extintores COT=$33.80 vs DB=$97.70 (neto $-63.90) | Cantidad: 1 ext en COT vs 7 en DB | DB tiene +1×50lbCO2 que no aparece en COT ($45/ext) | DB tiene +1×20lbPQS que no aparece en COT ($20/ext) | DB tiene +3×5lbCO2 que no aparece en COT ($4/ext) | DB tiene +1×10lbPQS que no aparece en COT ($10/ext)</t>
+          <t>Cotización por venta de extintores / servicio, no mantenimiento</t>
         </is>
       </c>
       <c r="M67" s="5" t="inlineStr">
         <is>
-          <t>¿RETIRAR 1×50lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×20lbPQS de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 3×5lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×10lbPQS de BD? (o verificar si fue omitido en COT)</t>
+          <t>Informativo — no afecta la base de datos</t>
         </is>
       </c>
     </row>
@@ -3726,41 +3601,41 @@
       <c r="M68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B69" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1455 AMCA24 MALL DEL SUR.xlsx</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C69" s="8" t="inlineStr">
         <is>
           <t>AMCA24</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr"/>
-      <c r="E69" s="6" t="n">
+      <c r="D69" s="8" t="inlineStr"/>
+      <c r="E69" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F69" s="6" t="n"/>
-      <c r="G69" s="6" t="inlineStr"/>
-      <c r="H69" s="6" t="n"/>
-      <c r="I69" s="6" t="inlineStr">
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="inlineStr"/>
+      <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J69" s="7" t="inlineStr">
+      <c r="J69" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K69" s="7" t="inlineStr"/>
-      <c r="L69" s="7" t="inlineStr"/>
-      <c r="M69" s="7" t="inlineStr"/>
+      <c r="K69" s="9" t="inlineStr"/>
+      <c r="L69" s="9" t="inlineStr"/>
+      <c r="M69" s="9" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3988,184 +3863,184 @@
       <c r="M74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1453 GUSG50 MALL DEL SUR.xlsx</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>GUSG50</t>
         </is>
       </c>
-      <c r="D75" s="6" t="inlineStr"/>
-      <c r="E75" s="6" t="n">
+      <c r="D75" s="8" t="inlineStr"/>
+      <c r="E75" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="F75" s="6" t="n"/>
-      <c r="G75" s="6" t="inlineStr"/>
-      <c r="H75" s="6" t="n"/>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="F75" s="8" t="n"/>
+      <c r="G75" s="8" t="inlineStr"/>
+      <c r="H75" s="8" t="n"/>
+      <c r="I75" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J75" s="7" t="inlineStr">
+      <c r="J75" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K75" s="7" t="inlineStr"/>
-      <c r="L75" s="7" t="inlineStr"/>
-      <c r="M75" s="7" t="inlineStr"/>
+      <c r="K75" s="9" t="inlineStr"/>
+      <c r="L75" s="9" t="inlineStr"/>
+      <c r="M75" s="9" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1454 AMCA06 TERMINAL.xlsx</t>
         </is>
       </c>
-      <c r="C76" s="6" t="inlineStr">
+      <c r="C76" s="8" t="inlineStr">
         <is>
           <t>AMCA6</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr"/>
-      <c r="E76" s="6" t="n">
+      <c r="D76" s="8" t="inlineStr"/>
+      <c r="E76" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="6" t="inlineStr"/>
-      <c r="H76" s="6" t="n"/>
-      <c r="I76" s="6" t="inlineStr">
+      <c r="F76" s="8" t="n"/>
+      <c r="G76" s="8" t="inlineStr"/>
+      <c r="H76" s="8" t="n"/>
+      <c r="I76" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J76" s="7" t="inlineStr">
+      <c r="J76" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×5lbPQS@$2</t>
         </is>
       </c>
-      <c r="K76" s="7" t="inlineStr"/>
-      <c r="L76" s="7" t="inlineStr"/>
-      <c r="M76" s="7" t="inlineStr"/>
+      <c r="K76" s="9" t="inlineStr"/>
+      <c r="L76" s="9" t="inlineStr"/>
+      <c r="M76" s="9" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="inlineStr">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1460 R004 SAN MARINO.xlsx</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>R004 - SAN MARINO</t>
         </is>
       </c>
-      <c r="E77" s="4" t="n">
+      <c r="E77" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="F77" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="n">
-        <v>13.89</v>
-      </c>
-      <c r="I77" s="4" t="inlineStr">
+      <c r="F77" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
+      <c r="M77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>MAYO</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>COTIZACION1463 R010 ORELLANA.xlsx</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>R010 - FRANCISCO DE ORELLANA</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>418.7</v>
+      </c>
+      <c r="F78" s="6" t="n">
+        <v>448.1</v>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>RECARGA</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J77" s="5" t="inlineStr">
-        <is>
-          <t>2×50lbCO2@$20 + 3×5lbCO2@$2 + 2×10lbPQS@$4 + 1×2.5glnK@$8</t>
-        </is>
-      </c>
-      <c r="K77" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×2.5GLSTIPO K@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="L77" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$62.00 vs DB=$72.00 (neto $-10.00) | COT tiene +1×50lbCO2 que no está en DB (precio $20/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | DB tiene +1×75lbCO2 que no aparece en COT ($30/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M77" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×50lbCO2 a BD? ($20/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿RETIRAR 1×75lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>MAYO</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>COTIZACION1463 R010 ORELLANA.xlsx</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>R10</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>R010 - FRANCISCO DE ORELLANA</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="n">
-        <v>418.7</v>
-      </c>
-      <c r="F78" s="2" t="n">
-        <v>418.7</v>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>RECARGA</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J78" s="3" t="inlineStr"/>
-      <c r="K78" s="3" t="inlineStr"/>
-      <c r="L78" s="3" t="inlineStr"/>
-      <c r="M78" s="3" t="inlineStr"/>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>1×75lbCO2@$68 + 2×10lbCO2@$9 + 4×5lbCO2@$4 + 1×20lbPQS@$20 + 10×10lbPQS@$10 + 2×2.5glnK@$99</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>1×75lbCO2@$68 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbCO2@$9 + 1×20lbPQS@$20 + 1×20lbPQS@$20 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×2.5GLSTIPO K@$99 + 1×2.5GLSTIPO K@$99  [+MOVIL:$18.80 — GYE-ORELLANA]</t>
+        </is>
+      </c>
+      <c r="L78" s="7" t="inlineStr">
+        <is>
+          <t>Viáticos COT=$0.00 vs DB=$18.80 | (viáticos no detectados en líneas COT, posible formato) | Extintores COT=$418.70 vs DB=$429.30 (neto $-10.60) | COT tiene +1×10lbCO2 que no está en DB (precio $9/ext) | COT tiene +2×2.5glnK que no está en DB (precio $99/ext) | DB tiene +2×2.5GLSTIPO K que no aparece en COT ($99/ext) | DB tiene +1×20lbPQS que no aparece en COT ($20/ext)</t>
+        </is>
+      </c>
+      <c r="M78" s="7" t="inlineStr">
+        <is>
+          <t>¿AGREGAR 1×10lbCO2 a BD? ($9/ext) | ¿AGREGAR 2×2.5glnK a BD? ($99/ext) | ¿RETIRAR 2×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×20lbPQS de BD? (o verificar si fue omitido en COT)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4258,281 +4133,281 @@
       <c r="M80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="4" t="inlineStr">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1452 KFCK96 PORTETE.xlsx</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="C81" s="6" t="inlineStr">
         <is>
           <t>K96</t>
         </is>
       </c>
-      <c r="D81" s="4" t="inlineStr">
+      <c r="D81" s="6" t="inlineStr">
         <is>
           <t>K096 - PORTETE</t>
         </is>
       </c>
-      <c r="E81" s="4" t="n">
+      <c r="E81" s="6" t="n">
         <v>76</v>
       </c>
-      <c r="F81" s="4" t="n">
-        <v>86</v>
-      </c>
-      <c r="G81" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H81" s="4" t="n">
-        <v>11.63</v>
-      </c>
-      <c r="I81" s="4" t="inlineStr">
+      <c r="F81" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J81" s="5" t="inlineStr">
+      <c r="J81" s="7" t="inlineStr">
         <is>
           <t>2×50lbCO2@$20 + 4×5lbCO2@$2 + 2×20lbPQS@$8 + 3×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K81" s="5" t="inlineStr">
-        <is>
-          <t>1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×20lbPQS@$8 + 1×50lbCO2@$20 + 1×10lbPQS@$4 + 1×5lbCO2@$2 + 1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×20lbPQS@$8 + 1×20lbPQS@$8</t>
-        </is>
-      </c>
-      <c r="L81" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$76.00 vs DB=$86.00 (neto $-10.00) | COT tiene +1×5lbCO2 que no está en DB (precio $2/ext) | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | DB tiene +2×20lbPQS que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M81" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×5lbCO2 a BD? ($2/ext) | ¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿RETIRAR 2×20lbPQS de BD? (o verificar si fue omitido en COT)</t>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>1×50lbCO2@$20 + 1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×20lbPQS@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8</t>
+        </is>
+      </c>
+      <c r="L81" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$76.00 vs DB=$84.00 (neto $-8.00) | Cantidad: 11 ext en COT vs 12 en DB | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
+        </is>
+      </c>
+      <c r="M81" s="7" t="inlineStr">
+        <is>
+          <t>¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="inlineStr">
+      <c r="A82" s="6" t="inlineStr">
         <is>
           <t>MAYO</t>
         </is>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1464 R010 ORELLANA.xlsx</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C82" s="6" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="D82" s="4" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>R010 - FRANCISCO DE ORELLANA</t>
         </is>
       </c>
-      <c r="E82" s="4" t="n">
+      <c r="E82" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="F82" s="4" t="n">
-        <v>418.7</v>
-      </c>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="F82" s="6" t="n">
+        <v>448.1</v>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H82" s="4" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="I82" s="4" t="inlineStr">
+      <c r="H82" s="6" t="n">
+        <v>79.92</v>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J82" s="5" t="inlineStr">
+      <c r="J82" s="7" t="inlineStr">
         <is>
           <t>(sin líneas ext)</t>
         </is>
       </c>
-      <c r="K82" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$68 + 1×10lbCO2@$9 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×20lbPQS@$20 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×2.5GLSTIPO K@$99 + 1×2.5GLSTIPO K@$99  [+MOVIL:$18.80 — GYE-ORELLANA]</t>
-        </is>
-      </c>
-      <c r="L82" s="5" t="inlineStr">
-        <is>
-          <t>Viáticos COT=$0.00 vs DB=$18.80 | (viáticos no detectados en líneas COT, posible formato) | Extintores COT=$0.00 vs DB=$399.90 (neto $-399.90) | Cantidad: 0 ext en COT vs 18 en DB | DB tiene +1×10lbCO2 que no aparece en COT ($9/ext) | DB tiene +2×2.5GLSTIPO K que no aparece en COT ($99/ext) | DB tiene +1×20lbPQS que no aparece en COT ($20/ext) | DB tiene +4×5lbCO2 que no aparece en COT ($4/ext) | DB tiene +9×10lbPQS que no aparece en COT ($10/ext) | DB tiene +1×75lbCO2 que no aparece en COT ($68/ext)</t>
-        </is>
-      </c>
-      <c r="M82" s="5" t="inlineStr">
-        <is>
-          <t>¿RETIRAR 1×10lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 2×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×20lbPQS de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 4×5lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 9×10lbPQS de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×75lbCO2 de BD? (o verificar si fue omitido en COT)</t>
+      <c r="K82" s="7" t="inlineStr">
+        <is>
+          <t>1×75lbCO2@$68 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbCO2@$9 + 1×20lbPQS@$20 + 1×20lbPQS@$20 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×2.5GLSTIPO K@$99 + 1×2.5GLSTIPO K@$99  [+MOVIL:$18.80 — GYE-ORELLANA]</t>
+        </is>
+      </c>
+      <c r="L82" s="7" t="inlineStr">
+        <is>
+          <t>Viáticos COT=$0.00 vs DB=$18.80 | (viáticos no detectados en líneas COT, posible formato) | Extintores COT=$0.00 vs DB=$429.30 (neto $-429.30) | Cantidad: 0 ext en COT vs 20 en DB | DB tiene +1×75lbCO2 que no aparece en COT ($68/ext) | DB tiene +2×2.5GLSTIPO K que no aparece en COT ($99/ext) | DB tiene +10×10lbPQS que no aparece en COT ($10/ext) | DB tiene +4×5lbCO2 que no aparece en COT ($4/ext) | DB tiene +1×10lbCO2 que no aparece en COT ($9/ext) | DB tiene +2×20lbPQS que no aparece en COT ($20/ext)</t>
+        </is>
+      </c>
+      <c r="M82" s="7" t="inlineStr">
+        <is>
+          <t>¿RETIRAR 1×75lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 2×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 10×10lbPQS de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 4×5lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×10lbCO2 de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 2×20lbPQS de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="inlineStr">
+      <c r="A83" s="8" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B83" s="6" t="inlineStr">
+      <c r="B83" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1501 ILCI04 MALL DEL SUR.xlsx</t>
         </is>
       </c>
-      <c r="C83" s="6" t="inlineStr">
+      <c r="C83" s="8" t="inlineStr">
         <is>
           <t>ILCI4</t>
         </is>
       </c>
-      <c r="D83" s="6" t="inlineStr"/>
-      <c r="E83" s="6" t="n">
+      <c r="D83" s="8" t="inlineStr"/>
+      <c r="E83" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="F83" s="6" t="n"/>
-      <c r="G83" s="6" t="inlineStr"/>
-      <c r="H83" s="6" t="n"/>
-      <c r="I83" s="6" t="inlineStr">
+      <c r="F83" s="8" t="n"/>
+      <c r="G83" s="8" t="inlineStr"/>
+      <c r="H83" s="8" t="n"/>
+      <c r="I83" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J83" s="7" t="inlineStr">
+      <c r="J83" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K83" s="7" t="inlineStr"/>
-      <c r="L83" s="7" t="inlineStr"/>
-      <c r="M83" s="7" t="inlineStr"/>
+      <c r="K83" s="9" t="inlineStr"/>
+      <c r="L83" s="9" t="inlineStr"/>
+      <c r="M83" s="9" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1511 F003 DOLCE INCONTRO  AEROPUERTO.xlsx</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" s="6" t="inlineStr">
         <is>
           <t>F3</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
+      <c r="D84" s="6" t="inlineStr">
         <is>
           <t>F003 - DOLCE INCONTRO AERGYE</t>
         </is>
       </c>
-      <c r="E84" s="4" t="n">
+      <c r="E84" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="F84" s="4" t="n">
+      <c r="F84" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="n">
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="n">
         <v>10.53</v>
       </c>
-      <c r="I84" s="4" t="inlineStr">
+      <c r="I84" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J84" s="5" t="inlineStr">
+      <c r="J84" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 3×10lbPQS@$4 + 1×2.5glnK@$8</t>
         </is>
       </c>
-      <c r="K84" s="5" t="inlineStr">
+      <c r="K84" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8</t>
         </is>
       </c>
-      <c r="L84" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$42.00 vs DB=$38.00 (neto +$4.00) | Cantidad: 6 ext en COT vs 5 en DB | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M84" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
+      <c r="L84" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$42.00 vs DB=$38.00 (neto +$4.00) | Cantidad: 6 ext en COT vs 5 en DB | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
+        </is>
+      </c>
+      <c r="M84" s="7" t="inlineStr">
+        <is>
+          <t>¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="inlineStr">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1507 CJNC08 TERMINAL.xlsx</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="C85" s="6" t="inlineStr">
         <is>
           <t>J8</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr">
+      <c r="D85" s="6" t="inlineStr">
         <is>
           <t>J008 - TERMINAL</t>
         </is>
       </c>
-      <c r="E85" s="4" t="n">
+      <c r="E85" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="F85" s="4" t="n">
+      <c r="F85" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H85" s="4" t="n">
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="n">
         <v>26.32</v>
       </c>
-      <c r="I85" s="4" t="inlineStr">
+      <c r="I85" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J85" s="5" t="inlineStr">
+      <c r="J85" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K85" s="5" t="inlineStr">
+      <c r="K85" s="7" t="inlineStr">
         <is>
           <t>1×75lbCO2@$30 + 1×10lbPQS@$4 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="L85" s="5" t="inlineStr">
+      <c r="L85" s="7" t="inlineStr">
         <is>
           <t>Extintores COT=$28.00 vs DB=$38.00 (neto $-10.00) | COT tiene +1×50lbCO2 que no está en DB (precio $20/ext) | DB tiene +1×75lbCO2 que no aparece en COT ($30/ext)</t>
         </is>
       </c>
-      <c r="M85" s="5" t="inlineStr">
+      <c r="M85" s="7" t="inlineStr">
         <is>
           <t>¿AGREGAR 1×50lbCO2 a BD? ($20/ext) | ¿RETIRAR 1×75lbCO2 de BD? (o verificar si fue omitido en COT)</t>
         </is>
@@ -4629,65 +4504,49 @@
       <c r="M87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1512 KFCK83 MUCHO LOTE.xlsx</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>K83</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>K083 - MUCHO LOTE</t>
         </is>
       </c>
-      <c r="E88" s="4" t="n">
+      <c r="E88" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="F88" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="G88" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H88" s="4" t="n">
-        <v>17.39</v>
-      </c>
-      <c r="I88" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J88" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 2×20lbPQS@$8 + 1×10lbPQS@$4</t>
-        </is>
-      </c>
-      <c r="K88" s="5" t="inlineStr">
-        <is>
-          <t>1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×20lbPQS@$8 + 1×75lbCO2@$30</t>
-        </is>
-      </c>
-      <c r="L88" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$54.00 vs DB=$46.00 (neto +$8.00) | Cantidad: 6 ext en COT vs 5 en DB | COT tiene +1×20lbPQS que no está en DB (precio $8/ext)</t>
-        </is>
-      </c>
-      <c r="M88" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×20lbPQS a BD? ($8/ext)</t>
-        </is>
-      </c>
+      <c r="F88" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="inlineStr"/>
+      <c r="M88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4780,78 +4639,78 @@
       <c r="M90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="6" t="inlineStr">
+      <c r="A91" s="8" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B91" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1504 GUSG52 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C91" s="6" t="inlineStr">
+      <c r="C91" s="8" t="inlineStr">
         <is>
           <t>GUSG52</t>
         </is>
       </c>
-      <c r="D91" s="6" t="inlineStr"/>
-      <c r="E91" s="6" t="n">
+      <c r="D91" s="8" t="inlineStr"/>
+      <c r="E91" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F91" s="6" t="n"/>
-      <c r="G91" s="6" t="inlineStr"/>
-      <c r="H91" s="6" t="n"/>
-      <c r="I91" s="6" t="inlineStr">
+      <c r="F91" s="8" t="n"/>
+      <c r="G91" s="8" t="inlineStr"/>
+      <c r="H91" s="8" t="n"/>
+      <c r="I91" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J91" s="7" t="inlineStr">
+      <c r="J91" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K91" s="7" t="inlineStr"/>
-      <c r="L91" s="7" t="inlineStr"/>
-      <c r="M91" s="7" t="inlineStr"/>
+      <c r="K91" s="9" t="inlineStr"/>
+      <c r="L91" s="9" t="inlineStr"/>
+      <c r="M91" s="9" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="inlineStr">
+      <c r="A92" s="8" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="B92" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1503 GUSG48 TERMINAL.xlsx</t>
         </is>
       </c>
-      <c r="C92" s="6" t="inlineStr">
+      <c r="C92" s="8" t="inlineStr">
         <is>
           <t>GUSG48</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr"/>
-      <c r="E92" s="6" t="n">
+      <c r="D92" s="8" t="inlineStr"/>
+      <c r="E92" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F92" s="6" t="n"/>
-      <c r="G92" s="6" t="inlineStr"/>
-      <c r="H92" s="6" t="n"/>
-      <c r="I92" s="6" t="inlineStr">
+      <c r="F92" s="8" t="n"/>
+      <c r="G92" s="8" t="inlineStr"/>
+      <c r="H92" s="8" t="n"/>
+      <c r="I92" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J92" s="7" t="inlineStr">
+      <c r="J92" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K92" s="7" t="inlineStr"/>
-      <c r="L92" s="7" t="inlineStr"/>
-      <c r="M92" s="7" t="inlineStr"/>
+      <c r="K92" s="9" t="inlineStr"/>
+      <c r="L92" s="9" t="inlineStr"/>
+      <c r="M92" s="9" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4899,65 +4758,49 @@
       <c r="M93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>JUNIO</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>COTIZACION1500 KFCK79 MALECON BABAHOYO.xlsx</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>K79</t>
         </is>
       </c>
-      <c r="D94" s="4" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>K079 - BABAHOYO</t>
         </is>
       </c>
-      <c r="E94" s="4" t="n">
+      <c r="E94" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="F94" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="G94" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H94" s="4" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="I94" s="4" t="inlineStr">
-        <is>
-          <t>INCONSISTENCIA</t>
-        </is>
-      </c>
-      <c r="J94" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 2×10lbCO2@$4 + 2×10lbPQS@$4  [+MOVIL:$40.00 — MOVILZIACION GYE - BABAHOYO(75KM)]</t>
-        </is>
-      </c>
-      <c r="K94" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4  [+MOVIL:$40.00 — GYE-BABAHOYO 75KM]</t>
-        </is>
-      </c>
-      <c r="L94" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$36.00 vs DB=$32.00 (neto +$4.00) | Cantidad: 5 ext en COT vs 4 en DB | COT tiene +1×10lbCO2 que no está en DB (precio $4/ext)</t>
-        </is>
-      </c>
-      <c r="M94" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbCO2 a BD? ($4/ext)</t>
-        </is>
-      </c>
+      <c r="F94" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr"/>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="inlineStr"/>
+      <c r="M94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5050,41 +4893,41 @@
       <c r="M96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="inlineStr">
+      <c r="A97" s="8" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B97" s="6" t="inlineStr">
+      <c r="B97" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1562 DOLCEI02 RIOC CEIBOS.xlsx</t>
         </is>
       </c>
-      <c r="C97" s="6" t="inlineStr">
+      <c r="C97" s="8" t="inlineStr">
         <is>
           <t>DOLCEI2</t>
         </is>
       </c>
-      <c r="D97" s="6" t="inlineStr"/>
-      <c r="E97" s="6" t="n">
+      <c r="D97" s="8" t="inlineStr"/>
+      <c r="E97" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="F97" s="6" t="n"/>
-      <c r="G97" s="6" t="inlineStr"/>
-      <c r="H97" s="6" t="n"/>
-      <c r="I97" s="6" t="inlineStr">
+      <c r="F97" s="8" t="n"/>
+      <c r="G97" s="8" t="inlineStr"/>
+      <c r="H97" s="8" t="n"/>
+      <c r="I97" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J97" s="7" t="inlineStr">
+      <c r="J97" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K97" s="7" t="inlineStr"/>
-      <c r="L97" s="7" t="inlineStr"/>
-      <c r="M97" s="7" t="inlineStr"/>
+      <c r="K97" s="9" t="inlineStr"/>
+      <c r="L97" s="9" t="inlineStr"/>
+      <c r="M97" s="9" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5222,41 +5065,41 @@
       <c r="M100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="6" t="inlineStr">
+      <c r="A101" s="8" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B101" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1563 DOLCEI03 RIOC ENTRE RIOS.xlsx</t>
         </is>
       </c>
-      <c r="C101" s="6" t="inlineStr">
+      <c r="C101" s="8" t="inlineStr">
         <is>
           <t>DOLCEI3</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr"/>
-      <c r="E101" s="6" t="n">
+      <c r="D101" s="8" t="inlineStr"/>
+      <c r="E101" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F101" s="6" t="n"/>
-      <c r="G101" s="6" t="inlineStr"/>
-      <c r="H101" s="6" t="n"/>
-      <c r="I101" s="6" t="inlineStr">
+      <c r="F101" s="8" t="n"/>
+      <c r="G101" s="8" t="inlineStr"/>
+      <c r="H101" s="8" t="n"/>
+      <c r="I101" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J101" s="7" t="inlineStr">
+      <c r="J101" s="9" t="inlineStr">
         <is>
           <t>1×10lbCO2@$4 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K101" s="7" t="inlineStr"/>
-      <c r="L101" s="7" t="inlineStr"/>
-      <c r="M101" s="7" t="inlineStr"/>
+      <c r="K101" s="9" t="inlineStr"/>
+      <c r="L101" s="9" t="inlineStr"/>
+      <c r="M101" s="9" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5304,41 +5147,41 @@
       <c r="M102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="6" t="inlineStr">
+      <c r="A103" s="8" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B103" s="6" t="inlineStr">
+      <c r="B103" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1552 GUSG47 ALBORADA.xlsx</t>
         </is>
       </c>
-      <c r="C103" s="6" t="inlineStr">
+      <c r="C103" s="8" t="inlineStr">
         <is>
           <t>GUSG47</t>
         </is>
       </c>
-      <c r="D103" s="6" t="inlineStr"/>
-      <c r="E103" s="6" t="n">
+      <c r="D103" s="8" t="inlineStr"/>
+      <c r="E103" s="8" t="n">
         <v>58</v>
       </c>
-      <c r="F103" s="6" t="n"/>
-      <c r="G103" s="6" t="inlineStr"/>
-      <c r="H103" s="6" t="n"/>
-      <c r="I103" s="6" t="inlineStr">
+      <c r="F103" s="8" t="n"/>
+      <c r="G103" s="8" t="inlineStr"/>
+      <c r="H103" s="8" t="n"/>
+      <c r="I103" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J103" s="7" t="inlineStr">
+      <c r="J103" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$30 + 1×10lbCO2@$4 + 1×20lbPQS@$8 + 4×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K103" s="7" t="inlineStr"/>
-      <c r="L103" s="7" t="inlineStr"/>
-      <c r="M103" s="7" t="inlineStr"/>
+      <c r="K103" s="9" t="inlineStr"/>
+      <c r="L103" s="9" t="inlineStr"/>
+      <c r="M103" s="9" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5791,78 +5634,78 @@
       <c r="M113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="6" t="inlineStr">
+      <c r="A114" s="8" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B114" s="6" t="inlineStr">
+      <c r="B114" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1556 AMCA07 SAN MARINO.xlsx</t>
         </is>
       </c>
-      <c r="C114" s="6" t="inlineStr">
+      <c r="C114" s="8" t="inlineStr">
         <is>
           <t>AMCA7</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr"/>
-      <c r="E114" s="6" t="n">
+      <c r="D114" s="8" t="inlineStr"/>
+      <c r="E114" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="F114" s="6" t="n"/>
-      <c r="G114" s="6" t="inlineStr"/>
-      <c r="H114" s="6" t="n"/>
-      <c r="I114" s="6" t="inlineStr">
+      <c r="F114" s="8" t="n"/>
+      <c r="G114" s="8" t="inlineStr"/>
+      <c r="H114" s="8" t="n"/>
+      <c r="I114" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J114" s="7" t="inlineStr">
+      <c r="J114" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×20lbPQS@$8 + 1×2.5glnK@$8</t>
         </is>
       </c>
-      <c r="K114" s="7" t="inlineStr"/>
-      <c r="L114" s="7" t="inlineStr"/>
-      <c r="M114" s="7" t="inlineStr"/>
+      <c r="K114" s="9" t="inlineStr"/>
+      <c r="L114" s="9" t="inlineStr"/>
+      <c r="M114" s="9" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="6" t="inlineStr">
+      <c r="A115" s="8" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B115" s="6" t="inlineStr">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1557 AMCA20 VILLAGE PLAZA.xlsx</t>
         </is>
       </c>
-      <c r="C115" s="6" t="inlineStr">
+      <c r="C115" s="8" t="inlineStr">
         <is>
           <t>AMCA20</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr"/>
-      <c r="E115" s="6" t="n">
+      <c r="D115" s="8" t="inlineStr"/>
+      <c r="E115" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="F115" s="6" t="n"/>
-      <c r="G115" s="6" t="inlineStr"/>
-      <c r="H115" s="6" t="n"/>
-      <c r="I115" s="6" t="inlineStr">
+      <c r="F115" s="8" t="n"/>
+      <c r="G115" s="8" t="inlineStr"/>
+      <c r="H115" s="8" t="n"/>
+      <c r="I115" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J115" s="7" t="inlineStr">
+      <c r="J115" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 3×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K115" s="7" t="inlineStr"/>
-      <c r="L115" s="7" t="inlineStr"/>
-      <c r="M115" s="7" t="inlineStr"/>
+      <c r="K115" s="9" t="inlineStr"/>
+      <c r="L115" s="9" t="inlineStr"/>
+      <c r="M115" s="9" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5910,124 +5753,124 @@
       <c r="M116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="4" t="inlineStr">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1574 KFCK162 SHELL PASCUALES.xlsx</t>
         </is>
       </c>
-      <c r="C117" s="4" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>K162</t>
         </is>
       </c>
-      <c r="D117" s="4" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>K162 - DAULE ESTACION</t>
         </is>
       </c>
-      <c r="E117" s="4" t="n">
+      <c r="E117" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="F117" s="4" t="n">
+      <c r="F117" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="G117" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H117" s="4" t="n">
+      <c r="G117" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H117" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="I117" s="4" t="inlineStr">
+      <c r="I117" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J117" s="5" t="inlineStr">
+      <c r="J117" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 3×5lbCO2@$2 + 1×10lbPQS@$4 + 2×10lbPQS@$4 + 1×2.5glnK@$8</t>
         </is>
       </c>
-      <c r="K117" s="5" t="inlineStr">
+      <c r="K117" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×5lbCO2@$2 + 1×20lbPQS@$8 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8</t>
         </is>
       </c>
-      <c r="L117" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$46.00 vs DB=$50.00 (neto $-4.00) | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | DB tiene +1×20lbPQS que no aparece en COT ($8/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext)</t>
-        </is>
-      </c>
-      <c r="M117" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿RETIRAR 1×20lbPQS de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT)</t>
+      <c r="L117" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$46.00 vs DB=$50.00 (neto $-4.00) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext) | DB tiene +1×20lbPQS que no aparece en COT ($8/ext)</t>
+        </is>
+      </c>
+      <c r="M117" s="7" t="inlineStr">
+        <is>
+          <t>¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 1×20lbPQS de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="4" t="inlineStr">
+      <c r="A118" s="6" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B118" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1575 KFCK171 SHELL ABUDHABI.xlsx</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr">
+      <c r="C118" s="6" t="inlineStr">
         <is>
           <t>K171</t>
         </is>
       </c>
-      <c r="D118" s="4" t="inlineStr">
+      <c r="D118" s="6" t="inlineStr">
         <is>
           <t>K171 - SHELL ABU DABI</t>
         </is>
       </c>
-      <c r="E118" s="4" t="n">
+      <c r="E118" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="F118" s="4" t="n">
+      <c r="F118" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="G118" s="4" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="H118" s="4" t="n">
+      <c r="G118" s="6" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="H118" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I118" s="4" t="inlineStr">
+      <c r="I118" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J118" s="5" t="inlineStr">
+      <c r="J118" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×10lbCO2@$4 + 1×20lbPQS@$8 + 1×2.5glnK@$8</t>
         </is>
       </c>
-      <c r="K118" s="5" t="inlineStr">
+      <c r="K118" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 1×10lbPQS@$4 + 1×10lbPQS@$4 + 1×2.5GLSTIPO K@$8</t>
         </is>
       </c>
-      <c r="L118" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$44.00 vs DB=$40.00 (neto +$4.00) | COT tiene +1×10lbCO2 que no está en DB (precio $4/ext) | COT tiene +1×20lbPQS que no está en DB (precio $8/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext) | DB tiene +2×10lbPQS que no aparece en COT ($4/ext)</t>
-        </is>
-      </c>
-      <c r="M118" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbCO2 a BD? ($4/ext) | ¿AGREGAR 1×20lbPQS a BD? ($8/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 2×10lbPQS de BD? (o verificar si fue omitido en COT)</t>
+      <c r="L118" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$44.00 vs DB=$40.00 (neto +$4.00) | COT tiene +1×10lbCO2 que no está en DB (precio $4/ext) | COT tiene +1×2.5glnK que no está en DB (precio $8/ext) | COT tiene +1×20lbPQS que no está en DB (precio $8/ext) | DB tiene +1×2.5GLSTIPO K que no aparece en COT ($8/ext) | DB tiene +2×10lbPQS que no aparece en COT ($4/ext)</t>
+        </is>
+      </c>
+      <c r="M118" s="7" t="inlineStr">
+        <is>
+          <t>¿AGREGAR 1×10lbCO2 a BD? ($4/ext) | ¿AGREGAR 1×2.5glnK a BD? ($8/ext) | ¿AGREGAR 1×20lbPQS a BD? ($8/ext) | ¿RETIRAR 1×2.5GLSTIPO K de BD? (o verificar si fue omitido en COT) | ¿RETIRAR 2×10lbPQS de BD? (o verificar si fue omitido en COT)</t>
         </is>
       </c>
     </row>
@@ -6077,41 +5920,41 @@
       <c r="M119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="6" t="inlineStr">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t>JULIO</t>
         </is>
       </c>
-      <c r="B120" s="6" t="inlineStr">
+      <c r="B120" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1571 GUSG51 SHOPPING QUEVEDO.xlsx</t>
         </is>
       </c>
-      <c r="C120" s="6" t="inlineStr">
+      <c r="C120" s="8" t="inlineStr">
         <is>
           <t>GUSG51</t>
         </is>
       </c>
-      <c r="D120" s="6" t="inlineStr"/>
-      <c r="E120" s="6" t="n">
+      <c r="D120" s="8" t="inlineStr"/>
+      <c r="E120" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="F120" s="6" t="n"/>
-      <c r="G120" s="6" t="inlineStr"/>
-      <c r="H120" s="6" t="n"/>
-      <c r="I120" s="6" t="inlineStr">
+      <c r="F120" s="8" t="n"/>
+      <c r="G120" s="8" t="inlineStr"/>
+      <c r="H120" s="8" t="n"/>
+      <c r="I120" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J120" s="7" t="inlineStr">
+      <c r="J120" s="9" t="inlineStr">
         <is>
           <t>1×75lbCO2@$30 + 1×5lbCO2@$2 + 1×10lbPQS@$4  [+MOVIL:$35.00 — MOVILIZACION (GUAYAQUIL-QUEVEDO)]</t>
         </is>
       </c>
-      <c r="K120" s="7" t="inlineStr"/>
-      <c r="L120" s="7" t="inlineStr"/>
-      <c r="M120" s="7" t="inlineStr"/>
+      <c r="K120" s="9" t="inlineStr"/>
+      <c r="L120" s="9" t="inlineStr"/>
+      <c r="M120" s="9" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6204,41 +6047,41 @@
       <c r="M122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="6" t="inlineStr">
+      <c r="A123" s="8" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="B123" s="6" t="inlineStr">
+      <c r="B123" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1614 ESPE22 AEROPUERTO ARRIBO NAC.xlsx</t>
         </is>
       </c>
-      <c r="C123" s="6" t="inlineStr">
+      <c r="C123" s="8" t="inlineStr">
         <is>
           <t>ESPE22</t>
         </is>
       </c>
-      <c r="D123" s="6" t="inlineStr"/>
-      <c r="E123" s="6" t="n">
+      <c r="D123" s="8" t="inlineStr"/>
+      <c r="E123" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F123" s="6" t="n"/>
-      <c r="G123" s="6" t="inlineStr"/>
-      <c r="H123" s="6" t="n"/>
-      <c r="I123" s="6" t="inlineStr">
+      <c r="F123" s="8" t="n"/>
+      <c r="G123" s="8" t="inlineStr"/>
+      <c r="H123" s="8" t="n"/>
+      <c r="I123" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J123" s="7" t="inlineStr">
+      <c r="J123" s="9" t="inlineStr">
         <is>
           <t>1×5lbCO2@$2 + 2×5lbPQS@$2</t>
         </is>
       </c>
-      <c r="K123" s="7" t="inlineStr"/>
-      <c r="L123" s="7" t="inlineStr"/>
-      <c r="M123" s="7" t="inlineStr"/>
+      <c r="K123" s="9" t="inlineStr"/>
+      <c r="L123" s="9" t="inlineStr"/>
+      <c r="M123" s="9" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6556,41 +6399,41 @@
       <c r="M130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" s="6" t="inlineStr">
+      <c r="A131" s="8" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="B131" s="6" t="inlineStr">
+      <c r="B131" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1609 AMCA19 MALL DEL SOL.xlsx</t>
         </is>
       </c>
-      <c r="C131" s="6" t="inlineStr">
+      <c r="C131" s="8" t="inlineStr">
         <is>
           <t>AMCA19</t>
         </is>
       </c>
-      <c r="D131" s="6" t="inlineStr"/>
-      <c r="E131" s="6" t="n">
+      <c r="D131" s="8" t="inlineStr"/>
+      <c r="E131" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="F131" s="6" t="n"/>
-      <c r="G131" s="6" t="inlineStr"/>
-      <c r="H131" s="6" t="n"/>
-      <c r="I131" s="6" t="inlineStr">
+      <c r="F131" s="8" t="n"/>
+      <c r="G131" s="8" t="inlineStr"/>
+      <c r="H131" s="8" t="n"/>
+      <c r="I131" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J131" s="7" t="inlineStr">
+      <c r="J131" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×10lbCO2@$4</t>
         </is>
       </c>
-      <c r="K131" s="7" t="inlineStr"/>
-      <c r="L131" s="7" t="inlineStr"/>
-      <c r="M131" s="7" t="inlineStr"/>
+      <c r="K131" s="9" t="inlineStr"/>
+      <c r="L131" s="9" t="inlineStr"/>
+      <c r="M131" s="9" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6863,41 +6706,41 @@
       <c r="M137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="6" t="inlineStr">
+      <c r="A138" s="8" t="inlineStr">
         <is>
           <t>AGOSTO</t>
         </is>
       </c>
-      <c r="B138" s="6" t="inlineStr">
+      <c r="B138" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1610 ESPE07 URDESA.xlsx</t>
         </is>
       </c>
-      <c r="C138" s="6" t="inlineStr">
+      <c r="C138" s="8" t="inlineStr">
         <is>
           <t>ESPE7</t>
         </is>
       </c>
-      <c r="D138" s="6" t="inlineStr"/>
-      <c r="E138" s="6" t="n">
+      <c r="D138" s="8" t="inlineStr"/>
+      <c r="E138" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="F138" s="6" t="n"/>
-      <c r="G138" s="6" t="inlineStr"/>
-      <c r="H138" s="6" t="n"/>
-      <c r="I138" s="6" t="inlineStr">
+      <c r="F138" s="8" t="n"/>
+      <c r="G138" s="8" t="inlineStr"/>
+      <c r="H138" s="8" t="n"/>
+      <c r="I138" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J138" s="7" t="inlineStr">
+      <c r="J138" s="9" t="inlineStr">
         <is>
           <t>2×5lbCO2@$2 + 4×10lbPQS@$4 + 1×5lbPQS@$2</t>
         </is>
       </c>
-      <c r="K138" s="7" t="inlineStr"/>
-      <c r="L138" s="7" t="inlineStr"/>
-      <c r="M138" s="7" t="inlineStr"/>
+      <c r="K138" s="9" t="inlineStr"/>
+      <c r="L138" s="9" t="inlineStr"/>
+      <c r="M138" s="9" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -6945,41 +6788,41 @@
       <c r="M139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="6" t="inlineStr">
+      <c r="A140" s="8" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
-      <c r="B140" s="6" t="inlineStr">
+      <c r="B140" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1651 AMCA33 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C140" s="6" t="inlineStr">
+      <c r="C140" s="8" t="inlineStr">
         <is>
           <t>AMCA33</t>
         </is>
       </c>
-      <c r="D140" s="6" t="inlineStr"/>
-      <c r="E140" s="6" t="n">
+      <c r="D140" s="8" t="inlineStr"/>
+      <c r="E140" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="F140" s="6" t="n"/>
-      <c r="G140" s="6" t="inlineStr"/>
-      <c r="H140" s="6" t="n"/>
-      <c r="I140" s="6" t="inlineStr">
+      <c r="F140" s="8" t="n"/>
+      <c r="G140" s="8" t="inlineStr"/>
+      <c r="H140" s="8" t="n"/>
+      <c r="I140" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J140" s="7" t="inlineStr">
+      <c r="J140" s="9" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K140" s="7" t="inlineStr"/>
-      <c r="L140" s="7" t="inlineStr"/>
-      <c r="M140" s="7" t="inlineStr"/>
+      <c r="K140" s="9" t="inlineStr"/>
+      <c r="L140" s="9" t="inlineStr"/>
+      <c r="M140" s="9" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -7027,41 +6870,41 @@
       <c r="M141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="6" t="inlineStr">
+      <c r="A142" s="8" t="inlineStr">
         <is>
           <t>SEPTIEMBRE</t>
         </is>
       </c>
-      <c r="B142" s="6" t="inlineStr">
+      <c r="B142" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1653 ESPE31 POLICENTRO.xlsx</t>
         </is>
       </c>
-      <c r="C142" s="6" t="inlineStr">
+      <c r="C142" s="8" t="inlineStr">
         <is>
           <t>ESPE31</t>
         </is>
       </c>
-      <c r="D142" s="6" t="inlineStr"/>
-      <c r="E142" s="6" t="n">
+      <c r="D142" s="8" t="inlineStr"/>
+      <c r="E142" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F142" s="6" t="n"/>
-      <c r="G142" s="6" t="inlineStr"/>
-      <c r="H142" s="6" t="n"/>
-      <c r="I142" s="6" t="inlineStr">
+      <c r="F142" s="8" t="n"/>
+      <c r="G142" s="8" t="inlineStr"/>
+      <c r="H142" s="8" t="n"/>
+      <c r="I142" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J142" s="7" t="inlineStr">
+      <c r="J142" s="9" t="inlineStr">
         <is>
           <t>1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K142" s="7" t="inlineStr"/>
-      <c r="L142" s="7" t="inlineStr"/>
-      <c r="M142" s="7" t="inlineStr"/>
+      <c r="K142" s="9" t="inlineStr"/>
+      <c r="L142" s="9" t="inlineStr"/>
+      <c r="M142" s="9" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -7109,601 +6952,601 @@
       <c r="M143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="6" t="inlineStr">
+      <c r="A144" s="8" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B144" s="6" t="inlineStr">
+      <c r="B144" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1213 KFC OFICINAS CENTRO.xlsx</t>
         </is>
       </c>
-      <c r="C144" s="6" t="inlineStr">
+      <c r="C144" s="8" t="inlineStr">
         <is>
           <t>KFC</t>
         </is>
       </c>
-      <c r="D144" s="6" t="inlineStr"/>
-      <c r="E144" s="6" t="n">
+      <c r="D144" s="8" t="inlineStr"/>
+      <c r="E144" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="F144" s="6" t="n"/>
-      <c r="G144" s="6" t="inlineStr"/>
-      <c r="H144" s="6" t="n"/>
-      <c r="I144" s="6" t="inlineStr">
+      <c r="F144" s="8" t="n"/>
+      <c r="G144" s="8" t="inlineStr"/>
+      <c r="H144" s="8" t="n"/>
+      <c r="I144" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J144" s="7" t="inlineStr">
+      <c r="J144" s="9" t="inlineStr">
         <is>
           <t>1×10lbCO2@$4 + 4×5lbCO2@$2 + 12×10lbPQS@$4 + 1×5lbPQS@$2</t>
         </is>
       </c>
-      <c r="K144" s="7" t="inlineStr"/>
-      <c r="L144" s="7" t="inlineStr"/>
-      <c r="M144" s="7" t="inlineStr"/>
+      <c r="K144" s="9" t="inlineStr"/>
+      <c r="L144" s="9" t="inlineStr"/>
+      <c r="M144" s="9" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="8" t="inlineStr">
+      <c r="A145" s="10" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B145" s="8" t="inlineStr">
+      <c r="B145" s="10" t="inlineStr">
         <is>
           <t>COTIZACION1217 M33 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C145" s="8" t="inlineStr">
+      <c r="C145" s="10" t="inlineStr">
         <is>
           <t>M33</t>
         </is>
       </c>
-      <c r="D145" s="8" t="inlineStr">
+      <c r="D145" s="10" t="inlineStr">
         <is>
           <t>M033 - CITY MALL</t>
         </is>
       </c>
-      <c r="E145" s="8" t="n">
+      <c r="E145" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="F145" s="8" t="n">
+      <c r="F145" s="10" t="n">
         <v>63.8</v>
       </c>
-      <c r="G145" s="8" t="inlineStr">
+      <c r="G145" s="10" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H145" s="8" t="n">
+      <c r="H145" s="10" t="n">
         <v>56.11</v>
       </c>
-      <c r="I145" s="8" t="inlineStr">
+      <c r="I145" s="10" t="inlineStr">
         <is>
           <t>COT_DEBE_RECARGA</t>
         </is>
       </c>
-      <c r="J145" s="9" t="inlineStr">
+      <c r="J145" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K145" s="9" t="inlineStr">
+      <c r="K145" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10</t>
         </is>
       </c>
-      <c r="L145" s="9" t="inlineStr">
-        <is>
-          <t>⚠ COT usa precio MANTENIMIENTO ($28.00). Debería ser RECARGA ($63.80). | Extintores COT=$28.00 vs DB=$63.80 (neto $-35.80) | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 2×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
-        </is>
-      </c>
-      <c r="M145" s="9" t="inlineStr">
+      <c r="L145" s="11" t="inlineStr">
+        <is>
+          <t>⚠ COT usa precio MANTENIMIENTO ($28.00). Debería ser RECARGA ($63.80). | Extintores COT=$28.00 vs DB=$63.80 (neto $-35.80) | 1×10lbPQS: precio COT=$4 vs DB=$10/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 2×5lbCO2: precio COT=$2 vs DB=$4/ext</t>
+        </is>
+      </c>
+      <c r="M145" s="11" t="inlineStr">
         <is>
           <t>Reemitir cotización como RECARGA por $63.80</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="8" t="inlineStr">
+      <c r="A146" s="10" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B146" s="8" t="inlineStr">
+      <c r="B146" s="10" t="inlineStr">
         <is>
           <t>COTIZACION1218 CJNC11 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C146" s="8" t="inlineStr">
+      <c r="C146" s="10" t="inlineStr">
         <is>
           <t>J11</t>
         </is>
       </c>
-      <c r="D146" s="8" t="inlineStr">
+      <c r="D146" s="10" t="inlineStr">
         <is>
           <t>J011 - CITY MALL</t>
         </is>
       </c>
-      <c r="E146" s="8" t="n">
+      <c r="E146" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="F146" s="8" t="n">
+      <c r="F146" s="10" t="n">
         <v>63.8</v>
       </c>
-      <c r="G146" s="8" t="inlineStr">
+      <c r="G146" s="10" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H146" s="8" t="n">
+      <c r="H146" s="10" t="n">
         <v>56.11</v>
       </c>
-      <c r="I146" s="8" t="inlineStr">
+      <c r="I146" s="10" t="inlineStr">
         <is>
           <t>COT_DEBE_RECARGA</t>
         </is>
       </c>
-      <c r="J146" s="9" t="inlineStr">
+      <c r="J146" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K146" s="9" t="inlineStr">
+      <c r="K146" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10</t>
         </is>
       </c>
-      <c r="L146" s="9" t="inlineStr">
-        <is>
-          <t>⚠ COT usa precio MANTENIMIENTO ($28.00). Debería ser RECARGA ($63.80). | Extintores COT=$28.00 vs DB=$63.80 (neto $-35.80) | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 2×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
-        </is>
-      </c>
-      <c r="M146" s="9" t="inlineStr">
+      <c r="L146" s="11" t="inlineStr">
+        <is>
+          <t>⚠ COT usa precio MANTENIMIENTO ($28.00). Debería ser RECARGA ($63.80). | Extintores COT=$28.00 vs DB=$63.80 (neto $-35.80) | 1×10lbPQS: precio COT=$4 vs DB=$10/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 2×5lbCO2: precio COT=$2 vs DB=$4/ext</t>
+        </is>
+      </c>
+      <c r="M146" s="11" t="inlineStr">
         <is>
           <t>Reemitir cotización como RECARGA por $63.80</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="6" t="inlineStr">
+      <c r="A147" s="8" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B147" s="6" t="inlineStr">
+      <c r="B147" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1219 ESPE09 RIOCENTRO CEIBOS.xlsx</t>
         </is>
       </c>
-      <c r="C147" s="6" t="inlineStr">
+      <c r="C147" s="8" t="inlineStr">
         <is>
           <t>ESPE9</t>
         </is>
       </c>
-      <c r="D147" s="6" t="inlineStr"/>
-      <c r="E147" s="6" t="n">
+      <c r="D147" s="8" t="inlineStr"/>
+      <c r="E147" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F147" s="6" t="n"/>
-      <c r="G147" s="6" t="inlineStr"/>
-      <c r="H147" s="6" t="n"/>
-      <c r="I147" s="6" t="inlineStr">
+      <c r="F147" s="8" t="n"/>
+      <c r="G147" s="8" t="inlineStr"/>
+      <c r="H147" s="8" t="n"/>
+      <c r="I147" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J147" s="7" t="inlineStr">
+      <c r="J147" s="9" t="inlineStr">
         <is>
           <t>1×5lbCO2@$2 + 1×10lbPQS@$4 + 1×5lbPQS@$2</t>
         </is>
       </c>
-      <c r="K147" s="7" t="inlineStr"/>
-      <c r="L147" s="7" t="inlineStr"/>
-      <c r="M147" s="7" t="inlineStr"/>
+      <c r="K147" s="9" t="inlineStr"/>
+      <c r="L147" s="9" t="inlineStr"/>
+      <c r="M147" s="9" t="inlineStr"/>
     </row>
     <row r="148">
-      <c r="A148" s="6" t="inlineStr">
+      <c r="A148" s="8" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B148" s="6" t="inlineStr">
+      <c r="B148" s="8" t="inlineStr">
         <is>
           <t>COTIZACION1220 ESPE30 CITY MALL.xlsx</t>
         </is>
       </c>
-      <c r="C148" s="6" t="inlineStr">
+      <c r="C148" s="8" t="inlineStr">
         <is>
           <t>ESPE30</t>
         </is>
       </c>
-      <c r="D148" s="6" t="inlineStr"/>
-      <c r="E148" s="6" t="n">
+      <c r="D148" s="8" t="inlineStr"/>
+      <c r="E148" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F148" s="6" t="n"/>
-      <c r="G148" s="6" t="inlineStr"/>
-      <c r="H148" s="6" t="n"/>
-      <c r="I148" s="6" t="inlineStr">
+      <c r="F148" s="8" t="n"/>
+      <c r="G148" s="8" t="inlineStr"/>
+      <c r="H148" s="8" t="n"/>
+      <c r="I148" s="8" t="inlineStr">
         <is>
           <t>SIN_MATCH_DB</t>
         </is>
       </c>
-      <c r="J148" s="7" t="inlineStr">
+      <c r="J148" s="9" t="inlineStr">
         <is>
           <t>1×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K148" s="7" t="inlineStr"/>
-      <c r="L148" s="7" t="inlineStr"/>
-      <c r="M148" s="7" t="inlineStr"/>
+      <c r="K148" s="9" t="inlineStr"/>
+      <c r="L148" s="9" t="inlineStr"/>
+      <c r="M148" s="9" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" s="8" t="inlineStr">
+      <c r="A149" s="10" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B149" s="8" t="inlineStr">
+      <c r="B149" s="10" t="inlineStr">
         <is>
           <t>COTIZACION1221 M61 PORTETE.xlsx</t>
         </is>
       </c>
-      <c r="C149" s="8" t="inlineStr">
+      <c r="C149" s="10" t="inlineStr">
         <is>
           <t>M61</t>
         </is>
       </c>
-      <c r="D149" s="8" t="inlineStr">
+      <c r="D149" s="10" t="inlineStr">
         <is>
           <t>M061 - PORTETE</t>
         </is>
       </c>
-      <c r="E149" s="8" t="n">
+      <c r="E149" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="F149" s="8" t="n">
+      <c r="F149" s="10" t="n">
         <v>152</v>
       </c>
-      <c r="G149" s="8" t="inlineStr">
+      <c r="G149" s="10" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H149" s="8" t="n">
+      <c r="H149" s="10" t="n">
         <v>57.89</v>
       </c>
-      <c r="I149" s="8" t="inlineStr">
+      <c r="I149" s="10" t="inlineStr">
         <is>
           <t>COT_DEBE_RECARGA</t>
         </is>
       </c>
-      <c r="J149" s="9" t="inlineStr">
+      <c r="J149" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 1×10lbCO2@$4 + 6×10lbPQS@$4 + 2×20lbPQS@$8</t>
         </is>
       </c>
-      <c r="K149" s="9" t="inlineStr">
+      <c r="K149" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$45 + 1×10lbCO2@$9 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×20lbPQS@$20 + 1×20lbPQS@$20</t>
         </is>
       </c>
-      <c r="L149" s="9" t="inlineStr">
-        <is>
-          <t>⚠ COT usa precio MANTENIMIENTO ($64.00). Debería ser RECARGA ($152.00). | Extintores COT=$64.00 vs DB=$152.00 (neto $-88.00) | 1×10lbCO2: precio COT=$4 vs DB=$9/ext | 2×20lbPQS: precio COT=$8 vs DB=$20/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 6×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
-        </is>
-      </c>
-      <c r="M149" s="9" t="inlineStr">
+      <c r="L149" s="11" t="inlineStr">
+        <is>
+          <t>⚠ COT usa precio MANTENIMIENTO ($64.00). Debería ser RECARGA ($152.00). | Extintores COT=$64.00 vs DB=$152.00 (neto $-88.00) | 1×10lbCO2: precio COT=$4 vs DB=$9/ext | 6×10lbPQS: precio COT=$4 vs DB=$10/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 2×20lbPQS: precio COT=$8 vs DB=$20/ext</t>
+        </is>
+      </c>
+      <c r="M149" s="11" t="inlineStr">
         <is>
           <t>Reemitir cotización como RECARGA por $152.00</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="8" t="inlineStr">
+      <c r="A150" s="10" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B150" s="8" t="inlineStr">
+      <c r="B150" s="10" t="inlineStr">
         <is>
           <t>COTIZACION1222 KFCK109 CITY MALL PA.xlsx</t>
         </is>
       </c>
-      <c r="C150" s="8" t="inlineStr">
+      <c r="C150" s="10" t="inlineStr">
         <is>
           <t>K109</t>
         </is>
       </c>
-      <c r="D150" s="8" t="inlineStr">
+      <c r="D150" s="10" t="inlineStr">
         <is>
           <t>K109 - CITY MALL PA</t>
         </is>
       </c>
-      <c r="E150" s="8" t="n">
+      <c r="E150" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="F150" s="8" t="n">
+      <c r="F150" s="10" t="n">
         <v>72.8</v>
       </c>
-      <c r="G150" s="8" t="inlineStr">
+      <c r="G150" s="10" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H150" s="8" t="n">
+      <c r="H150" s="10" t="n">
         <v>56.04</v>
       </c>
-      <c r="I150" s="8" t="inlineStr">
+      <c r="I150" s="10" t="inlineStr">
         <is>
           <t>COT_DEBE_RECARGA</t>
         </is>
       </c>
-      <c r="J150" s="9" t="inlineStr">
+      <c r="J150" s="11" t="inlineStr">
         <is>
           <t>1×50lb?@$20 + 1×10lbCO2@$4 + 2×5lbCO2@$2 + 1×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K150" s="9" t="inlineStr">
+      <c r="K150" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$45 + 1×10lbCO2@$9 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10</t>
         </is>
       </c>
-      <c r="L150" s="9" t="inlineStr">
-        <is>
-          <t>⚠ COT usa precio MANTENIMIENTO ($32.00). Debería ser RECARGA ($72.80). | Extintores COT=$32.00 vs DB=$72.80 (neto $-40.80) | COT tiene +1×50lb? que no está en DB (precio $20/ext) | DB tiene +1×50lbCO2 que no aparece en COT ($45/ext) | 1×10lbCO2: precio COT=$4 vs DB=$9/ext | 2×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
-        </is>
-      </c>
-      <c r="M150" s="9" t="inlineStr">
+      <c r="L150" s="11" t="inlineStr">
+        <is>
+          <t>⚠ COT usa precio MANTENIMIENTO ($32.00). Debería ser RECARGA ($72.80). | Extintores COT=$32.00 vs DB=$72.80 (neto $-40.80) | COT tiene +1×50lb? que no está en DB (precio $20/ext) | DB tiene +1×50lbCO2 que no aparece en COT ($45/ext) | 2×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×10lbCO2: precio COT=$4 vs DB=$9/ext | 1×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
+        </is>
+      </c>
+      <c r="M150" s="11" t="inlineStr">
         <is>
           <t>Reemitir cotización como RECARGA por $72.80</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="4" t="inlineStr">
+      <c r="A151" s="6" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B151" s="4" t="inlineStr">
+      <c r="B151" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1214 KFCK88 HIPER VIA A DAULE.xlsx</t>
         </is>
       </c>
-      <c r="C151" s="4" t="inlineStr">
+      <c r="C151" s="6" t="inlineStr">
         <is>
           <t>K88</t>
         </is>
       </c>
-      <c r="D151" s="4" t="inlineStr">
+      <c r="D151" s="6" t="inlineStr">
         <is>
           <t>K088 - HIPERMARKET VIA DAULE</t>
         </is>
       </c>
-      <c r="E151" s="4" t="n">
+      <c r="E151" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="F151" s="4" t="n">
+      <c r="F151" s="6" t="n">
         <v>97.7</v>
       </c>
-      <c r="G151" s="4" t="inlineStr">
+      <c r="G151" s="6" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H151" s="4" t="n">
+      <c r="H151" s="6" t="n">
         <v>52.92</v>
       </c>
-      <c r="I151" s="4" t="inlineStr">
+      <c r="I151" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J151" s="5" t="inlineStr">
+      <c r="J151" s="7" t="inlineStr">
         <is>
           <t>1×50lbCO2@$20 + 3×5lbCO2@$2 + 3×10lbPQS@$4 + 1×20lbPQS@$8</t>
         </is>
       </c>
-      <c r="K151" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×20lbPQS@$20</t>
-        </is>
-      </c>
-      <c r="L151" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$46.00 vs DB=$97.70 (neto $-51.70) | Cantidad: 8 ext en COT vs 7 en DB | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | 1×20lbPQS: precio COT=$8 vs DB=$20/ext | 3×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext</t>
-        </is>
-      </c>
-      <c r="M151" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿Actualizar precio 20lbPQS en BD: $20→$8/ext? | ¿Actualizar precio 5lbCO2 en BD: $4→$2/ext? | ¿Actualizar precio 50lbCO2 en BD: $45→$20/ext?</t>
+      <c r="K151" s="7" t="inlineStr">
+        <is>
+          <t>1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×20lbPQS@$20 + 1×10lbPQS@$10 + 1×10lbPQS@$10</t>
+        </is>
+      </c>
+      <c r="L151" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$46.00 vs DB=$97.70 (neto $-51.70) | Cantidad: 8 ext en COT vs 7 en DB | COT tiene +1×10lbPQS que no está en DB (precio $4/ext) | 3×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 1×20lbPQS: precio COT=$8 vs DB=$20/ext</t>
+        </is>
+      </c>
+      <c r="M151" s="7" t="inlineStr">
+        <is>
+          <t>¿AGREGAR 1×10lbPQS a BD? ($4/ext) | ¿Actualizar precio 5lbCO2 en BD: $4→$2/ext? | ¿Actualizar precio 50lbCO2 en BD: $45→$20/ext? | ¿Actualizar precio 20lbPQS en BD: $20→$8/ext?</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="4" t="inlineStr">
+      <c r="A152" s="6" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B152" s="4" t="inlineStr">
+      <c r="B152" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1215 KFCK110 CITY MALL PB.xlsx</t>
         </is>
       </c>
-      <c r="C152" s="4" t="inlineStr">
+      <c r="C152" s="6" t="inlineStr">
         <is>
           <t>K110</t>
         </is>
       </c>
-      <c r="D152" s="4" t="inlineStr">
+      <c r="D152" s="6" t="inlineStr">
         <is>
           <t>K110 - CITY MALL PB</t>
         </is>
       </c>
-      <c r="E152" s="4" t="n">
+      <c r="E152" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="F152" s="4" t="n">
+      <c r="F152" s="6" t="n">
         <v>124.7</v>
       </c>
-      <c r="G152" s="4" t="inlineStr">
+      <c r="G152" s="6" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H152" s="4" t="n">
+      <c r="H152" s="6" t="n">
         <v>59.9</v>
       </c>
-      <c r="I152" s="4" t="inlineStr">
+      <c r="I152" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J152" s="5" t="inlineStr">
+      <c r="J152" s="7" t="inlineStr">
         <is>
           <t>1×75lbCO2@$30 + 2×5lbCO2@$2 + 1×20lbPQS@$8 + 2×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K152" s="5" t="inlineStr">
-        <is>
-          <t>1×75lbCO2@$68 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×20lbPQS@$20 + 1×10lbCO2@$9 + 1×10lbPQS@$10 + 1×10lbPQS@$10</t>
-        </is>
-      </c>
-      <c r="L152" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$50.00 vs DB=$124.70 (neto $-74.70) | Cantidad: 6 ext en COT vs 7 en DB | DB tiene +1×10lbCO2 que no aparece en COT ($9/ext) | 1×75lbCO2: precio COT=$30 vs DB=$68/ext | 1×20lbPQS: precio COT=$8 vs DB=$20/ext | 2×5lbCO2: precio COT=$2 vs DB=$4/ext | 2×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
-        </is>
-      </c>
-      <c r="M152" s="5" t="inlineStr">
-        <is>
-          <t>¿RETIRAR 1×10lbCO2 de BD? (o verificar si fue omitido en COT) | ¿Actualizar precio 75lbCO2 en BD: $68→$30/ext? | ¿Actualizar precio 20lbPQS en BD: $20→$8/ext? | ¿Actualizar precio 5lbCO2 en BD: $4→$2/ext? | ¿Actualizar precio 10lbPQS en BD: $10→$4/ext?</t>
+      <c r="K152" s="7" t="inlineStr">
+        <is>
+          <t>1×75lbCO2@$68 + 1×10lbCO2@$9 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×20lbPQS@$20 + 1×10lbPQS@$10 + 1×10lbPQS@$10</t>
+        </is>
+      </c>
+      <c r="L152" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$50.00 vs DB=$124.70 (neto $-74.70) | Cantidad: 6 ext en COT vs 7 en DB | DB tiene +1×10lbCO2 que no aparece en COT ($9/ext) | 2×5lbCO2: precio COT=$2 vs DB=$4/ext | 1×75lbCO2: precio COT=$30 vs DB=$68/ext | 2×10lbPQS: precio COT=$4 vs DB=$10/ext | 1×20lbPQS: precio COT=$8 vs DB=$20/ext</t>
+        </is>
+      </c>
+      <c r="M152" s="7" t="inlineStr">
+        <is>
+          <t>¿RETIRAR 1×10lbCO2 de BD? (o verificar si fue omitido en COT) | ¿Actualizar precio 5lbCO2 en BD: $4→$2/ext? | ¿Actualizar precio 75lbCO2 en BD: $68→$30/ext? | ¿Actualizar precio 10lbPQS en BD: $10→$4/ext? | ¿Actualizar precio 20lbPQS en BD: $20→$8/ext?</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="8" t="inlineStr">
+      <c r="A153" s="10" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B153" s="8" t="inlineStr">
+      <c r="B153" s="10" t="inlineStr">
         <is>
           <t>COTIZACION1216 KFCK117 SEDALANA.xlsx</t>
         </is>
       </c>
-      <c r="C153" s="8" t="inlineStr">
+      <c r="C153" s="10" t="inlineStr">
         <is>
           <t>K117</t>
         </is>
       </c>
-      <c r="D153" s="8" t="inlineStr">
+      <c r="D153" s="10" t="inlineStr">
         <is>
           <t>K117 - 29 Y SEDALANA</t>
         </is>
       </c>
-      <c r="E153" s="8" t="n">
+      <c r="E153" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="F153" s="8" t="n">
+      <c r="F153" s="10" t="n">
         <v>241.2</v>
       </c>
-      <c r="G153" s="8" t="inlineStr">
+      <c r="G153" s="10" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H153" s="8" t="n">
+      <c r="H153" s="10" t="n">
         <v>56.88</v>
       </c>
-      <c r="I153" s="8" t="inlineStr">
+      <c r="I153" s="10" t="inlineStr">
         <is>
           <t>COT_DEBE_RECARGA</t>
         </is>
       </c>
-      <c r="J153" s="9" t="inlineStr">
+      <c r="J153" s="11" t="inlineStr">
         <is>
           <t>3×50lbCO2@$20 + 4×5lbCO2@$2 + 2×20lbPQS@$8 + 5×10lbPQS@$4</t>
         </is>
       </c>
-      <c r="K153" s="9" t="inlineStr">
+      <c r="K153" s="11" t="inlineStr">
         <is>
           <t>1×50lbCO2@$45 + 1×50lbCO2@$45 + 1×50lbCO2@$45 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×5lbCO2@$4 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×20lbPQS@$20 + 1×20lbPQS@$20 + 1×10lbPQS@$10</t>
         </is>
       </c>
-      <c r="L153" s="9" t="inlineStr">
-        <is>
-          <t>⚠ COT usa precio MANTENIMIENTO ($104.00). Debería ser RECARGA ($241.20). | Extintores COT=$104.00 vs DB=$241.20 (neto $-137.20) | 2×20lbPQS: precio COT=$8 vs DB=$20/ext | 4×5lbCO2: precio COT=$2 vs DB=$4/ext | 3×50lbCO2: precio COT=$20 vs DB=$45/ext | 5×10lbPQS: precio COT=$4 vs DB=$10/ext</t>
-        </is>
-      </c>
-      <c r="M153" s="9" t="inlineStr">
+      <c r="L153" s="11" t="inlineStr">
+        <is>
+          <t>⚠ COT usa precio MANTENIMIENTO ($104.00). Debería ser RECARGA ($241.20). | Extintores COT=$104.00 vs DB=$241.20 (neto $-137.20) | 4×5lbCO2: precio COT=$2 vs DB=$4/ext | 5×10lbPQS: precio COT=$4 vs DB=$10/ext | 3×50lbCO2: precio COT=$20 vs DB=$45/ext | 2×20lbPQS: precio COT=$8 vs DB=$20/ext</t>
+        </is>
+      </c>
+      <c r="M153" s="11" t="inlineStr">
         <is>
           <t>Reemitir cotización como RECARGA por $241.20</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="4" t="inlineStr">
+      <c r="A154" s="6" t="inlineStr">
         <is>
           <t>OCTUBRE</t>
         </is>
       </c>
-      <c r="B154" s="4" t="inlineStr">
+      <c r="B154" s="6" t="inlineStr">
         <is>
           <t>COTIZACION1212 B001 ARRECIFE AEROPUERTO.xlsx</t>
         </is>
       </c>
-      <c r="C154" s="4" t="inlineStr">
+      <c r="C154" s="6" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D154" s="4" t="inlineStr">
+      <c r="D154" s="6" t="inlineStr">
         <is>
           <t>B001 - STATION SPORTS BAR</t>
         </is>
       </c>
-      <c r="E154" s="4" t="n">
+      <c r="E154" s="6" t="n">
         <v>78.8</v>
       </c>
-      <c r="F154" s="4" t="n">
-        <v>92.40000000000001</v>
-      </c>
-      <c r="G154" s="4" t="inlineStr">
+      <c r="F154" s="6" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="G154" s="6" t="inlineStr">
         <is>
           <t>RECARGA</t>
         </is>
       </c>
-      <c r="H154" s="4" t="n">
-        <v>14.72</v>
-      </c>
-      <c r="I154" s="4" t="inlineStr">
+      <c r="H154" s="6" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="I154" s="6" t="inlineStr">
         <is>
           <t>INCONSISTENCIA</t>
         </is>
       </c>
-      <c r="J154" s="5" t="inlineStr">
+      <c r="J154" s="7" t="inlineStr">
         <is>
           <t>1×20lbCO2@$20 + 3×10lbPQS@$10 + 2×5lbPQS@$5 + 1×50lbCO2@$20</t>
         </is>
       </c>
-      <c r="K154" s="5" t="inlineStr">
-        <is>
-          <t>1×50lbCO2@$45 + 1×20lbCO2@$18 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10</t>
-        </is>
-      </c>
-      <c r="L154" s="5" t="inlineStr">
-        <is>
-          <t>Extintores COT=$78.80 vs DB=$92.40 (neto $-13.60) | Cantidad: 7 ext en COT vs 5 en DB | COT tiene +2×5lbPQS que no está en DB (precio $5/ext) | 1×50lbCO2: precio COT=$20 vs DB=$45/ext | 1×20lbCO2: precio COT=$20 vs DB=$18/ext</t>
-        </is>
-      </c>
-      <c r="M154" s="5" t="inlineStr">
-        <is>
-          <t>¿AGREGAR 2×5lbPQS a BD? ($5/ext) | ¿Actualizar precio 50lbCO2 en BD: $45→$20/ext? | ¿Actualizar precio 20lbCO2 en BD: $18→$20/ext?</t>
+      <c r="K154" s="7" t="inlineStr">
+        <is>
+          <t>1×50lbCO2@$45 + 1×20lbCO2@$18 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×10lbPQS@$10 + 1×5lbPQS@$5 + 1×5lbPQS@$5</t>
+        </is>
+      </c>
+      <c r="L154" s="7" t="inlineStr">
+        <is>
+          <t>Extintores COT=$78.80 vs DB=$102.20 (neto $-23.40) | 1×20lbCO2: precio COT=$20 vs DB=$18/ext | 1×50lbCO2: precio COT=$20 vs DB=$45/ext</t>
+        </is>
+      </c>
+      <c r="M154" s="7" t="inlineStr">
+        <is>
+          <t>¿Actualizar precio 20lbCO2 en BD: $18→$20/ext? | ¿Actualizar precio 50lbCO2 en BD: $45→$20/ext?</t>
         </is>
       </c>
     </row>
@@ -7726,7 +7569,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>RESUMEN REVISION COTIZACIONES 2026</t>
         </is>
@@ -7754,7 +7597,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5">
@@ -7764,7 +7607,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -7784,7 +7627,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -7847,10 +7690,10 @@
         <v>24</v>
       </c>
       <c r="C11" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -7859,7 +7702,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -7872,10 +7715,10 @@
         <v>20</v>
       </c>
       <c r="C12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -7897,10 +7740,10 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -7925,16 +7768,16 @@
         <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -7972,10 +7815,10 @@
         <v>13</v>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>

</xml_diff>